<commit_message>
actualizacion del gantt y visual
</commit_message>
<xml_diff>
--- a/VTT Tool/VTT DATA.xlsx
+++ b/VTT Tool/VTT DATA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOJorge\Documents\Python projects\Horse Luis\VTT Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B625301-F6F2-4413-8C13-0B4C7EBA3F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F679A5B8-B187-495D-BB0A-7ADF3FD61CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
   </bookViews>
@@ -365,7 +365,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="162">
   <si>
     <t>Compte Consignee</t>
   </si>
@@ -839,6 +839,18 @@
   </si>
   <si>
     <t>INFIMOTION</t>
+  </si>
+  <si>
+    <t>O001</t>
+  </si>
+  <si>
+    <t>MAERSK</t>
+  </si>
+  <si>
+    <t>DSV</t>
+  </si>
+  <si>
+    <t>WUHAN JINRUI TECH</t>
   </si>
 </sst>
 </file>
@@ -1013,7 +1025,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1059,10 +1071,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1076,7 +1084,7 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1137,7 +1145,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1453,11 +1461,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
-  <sheetPr codeName="Feuil4" filterMode="1">
+  <sheetPr codeName="Feuil4">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
-  <dimension ref="A1:BD51"/>
-  <sheetFormatPr defaultColWidth="10.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:BD52"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="5" width="10.42578125" customWidth="1"/>
     <col min="6" max="6" width="12.42578125" style="14" customWidth="1"/>
@@ -1481,180 +1489,180 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:56" ht="75" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="16" t="s">
+      <c r="E1" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="J1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="K1" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="L1" s="19" t="s">
+      <c r="L1" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="M1" s="19" t="s">
+      <c r="M1" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="N1" s="20" t="s">
+      <c r="N1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="21" t="s">
+      <c r="O1" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="P1" s="17" t="s">
+      <c r="P1" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="Q1" s="21" t="s">
+      <c r="Q1" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="R1" s="21" t="s">
+      <c r="R1" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="S1" s="21" t="s">
+      <c r="S1" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="T1" s="21" t="s">
+      <c r="T1" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="U1" s="17" t="s">
+      <c r="U1" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="V1" s="17" t="s">
+      <c r="V1" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="W1" s="17" t="s">
+      <c r="W1" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="X1" s="22" t="s">
+      <c r="X1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="Y1" s="22" t="s">
+      <c r="Y1" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="Z1" s="17" t="s">
+      <c r="Z1" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="AA1" s="17" t="s">
+      <c r="AA1" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="AB1" s="17" t="s">
+      <c r="AB1" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="AC1" s="34" t="s">
+      <c r="AC1" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="AD1" s="34" t="s">
+      <c r="AD1" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="AE1" s="17" t="s">
+      <c r="AE1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="AF1" s="17" t="s">
+      <c r="AF1" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="AG1" s="17" t="s">
+      <c r="AG1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="AH1" s="17" t="s">
+      <c r="AH1" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="AI1" s="17" t="s">
+      <c r="AI1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="AJ1" s="17" t="s">
+      <c r="AJ1" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="AK1" s="17" t="s">
+      <c r="AK1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="AL1" s="17" t="s">
+      <c r="AL1" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="AM1" s="17" t="s">
+      <c r="AM1" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="AN1" s="17" t="s">
+      <c r="AN1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="AO1" s="17" t="s">
+      <c r="AO1" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="AP1" s="17" t="s">
+      <c r="AP1" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="AQ1" s="17" t="s">
+      <c r="AQ1" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="AR1" s="17" t="s">
+      <c r="AR1" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="AS1" s="17" t="s">
+      <c r="AS1" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="AT1" s="23" t="s">
+      <c r="AT1" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="AU1" s="23" t="s">
+      <c r="AU1" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="AV1" s="34" t="s">
+      <c r="AV1" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="AW1" s="24" t="s">
+      <c r="AW1" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="AX1" s="17" t="s">
+      <c r="AX1" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="AY1" s="23" t="s">
+      <c r="AY1" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="AZ1" s="23" t="s">
+      <c r="AZ1" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="BA1" s="17" t="s">
+      <c r="BA1" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="BB1" s="17" t="s">
+      <c r="BB1" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="BC1" s="17" t="s">
+      <c r="BC1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="BD1" s="25" t="s">
+      <c r="BD1" s="24" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A2" s="6">
         <v>416</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="25" t="s">
         <v>77</v>
       </c>
       <c r="C2" s="7" t="s">
@@ -1666,7 +1674,7 @@
       <c r="E2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F2" s="27">
+      <c r="F2" s="26">
         <v>90014400</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -1833,18 +1841,18 @@
       <c r="BB2" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC2" s="28" t="s">
+      <c r="BC2" s="27" t="s">
         <v>82</v>
       </c>
-      <c r="BD2" s="29">
+      <c r="BD2" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="3" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A3" s="6">
         <v>901</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="25" t="s">
         <v>92</v>
       </c>
       <c r="C3" s="7" t="s">
@@ -1856,7 +1864,7 @@
       <c r="E3" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F3" s="27">
+      <c r="F3" s="26">
         <v>90012500</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -2023,18 +2031,18 @@
       <c r="BB3" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC3" s="28" t="s">
+      <c r="BC3" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD3" s="29">
+      <c r="BD3" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="4" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A4" s="6">
         <v>916</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="25" t="s">
         <v>96</v>
       </c>
       <c r="C4" s="7" t="s">
@@ -2046,7 +2054,7 @@
       <c r="E4" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="F4" s="27">
+      <c r="F4" s="26">
         <v>91017700</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -2213,18 +2221,18 @@
       <c r="BB4" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC4" s="28" t="s">
+      <c r="BC4" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD4" s="29">
+      <c r="BD4" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="5" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15">
+    <row r="5" spans="1:56" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
         <v>752</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="25" t="s">
         <v>83</v>
       </c>
       <c r="C5" s="7" t="s">
@@ -2236,7 +2244,7 @@
       <c r="E5" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F5" s="27">
+      <c r="F5" s="26">
         <v>90018000</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -2403,18 +2411,18 @@
       <c r="BB5" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC5" s="28" t="s">
+      <c r="BC5" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="BD5" s="29">
+      <c r="BD5" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="6" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>761</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="29" t="s">
         <v>86</v>
       </c>
       <c r="C6" s="7" t="s">
@@ -2426,7 +2434,7 @@
       <c r="E6" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="F6" s="27">
+      <c r="F6" s="26">
         <v>90016900</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -2593,18 +2601,18 @@
       <c r="BB6" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC6" s="28" t="s">
+      <c r="BC6" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="BD6" s="29">
+      <c r="BD6" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="7" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15">
+    <row r="7" spans="1:56" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
         <v>927</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="29" t="s">
         <v>77</v>
       </c>
       <c r="C7" s="7" t="s">
@@ -2616,7 +2624,7 @@
       <c r="E7" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F7" s="27">
+      <c r="F7" s="26">
         <v>90014400</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -2783,18 +2791,18 @@
       <c r="BB7" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC7" s="28" t="s">
+      <c r="BC7" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD7" s="29">
+      <c r="BD7" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="8" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A8" s="6">
         <v>930</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="30" t="s">
         <v>96</v>
       </c>
       <c r="C8" s="7" t="s">
@@ -2806,7 +2814,7 @@
       <c r="E8" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="F8" s="27">
+      <c r="F8" s="26">
         <v>91017700</v>
       </c>
       <c r="G8" s="9" t="s">
@@ -2973,18 +2981,18 @@
       <c r="BB8" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC8" s="28" t="s">
+      <c r="BC8" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD8" s="29">
+      <c r="BD8" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="9" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
         <v>931</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="29" t="s">
         <v>83</v>
       </c>
       <c r="C9" s="7" t="s">
@@ -2996,7 +3004,7 @@
       <c r="E9" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="F9" s="27">
+      <c r="F9" s="26">
         <v>90018600</v>
       </c>
       <c r="G9" s="11" t="s">
@@ -3005,7 +3013,7 @@
       <c r="H9" s="3">
         <v>26037000</v>
       </c>
-      <c r="I9" s="32" t="s">
+      <c r="I9" s="31" t="s">
         <v>48</v>
       </c>
       <c r="J9" s="3">
@@ -3163,18 +3171,18 @@
       <c r="BB9" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC9" s="28" t="s">
+      <c r="BC9" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD9" s="29">
+      <c r="BD9" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="10" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A10" s="6">
         <v>932</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="25" t="s">
         <v>92</v>
       </c>
       <c r="C10" s="7" t="s">
@@ -3186,7 +3194,7 @@
       <c r="E10" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="27">
+      <c r="F10" s="26">
         <v>90012500</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -3353,18 +3361,18 @@
       <c r="BB10" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC10" s="28" t="s">
+      <c r="BC10" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD10" s="29">
+      <c r="BD10" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="11" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+    <row r="11" spans="1:56" x14ac:dyDescent="0.25">
+      <c r="A11" s="6">
         <v>1027</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="29" t="s">
         <v>96</v>
       </c>
       <c r="C11" s="7" t="s">
@@ -3376,7 +3384,7 @@
       <c r="E11" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F11" s="27">
+      <c r="F11" s="26">
         <v>91017700</v>
       </c>
       <c r="G11" s="8" t="s">
@@ -3543,18 +3551,18 @@
       <c r="BB11" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC11" s="28" t="s">
+      <c r="BC11" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD11" s="29">
+      <c r="BD11" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="12" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
         <v>1045</v>
       </c>
-      <c r="B12" s="30" t="s">
+      <c r="B12" s="29" t="s">
         <v>77</v>
       </c>
       <c r="C12" s="7" t="s">
@@ -3566,7 +3574,7 @@
       <c r="E12" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F12" s="27">
+      <c r="F12" s="26">
         <v>90014400</v>
       </c>
       <c r="G12" s="8" t="s">
@@ -3733,18 +3741,18 @@
       <c r="BB12" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC12" s="28" t="s">
+      <c r="BC12" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="BD12" s="29">
+      <c r="BD12" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="13" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A13" s="6">
         <v>1060</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C13" s="7" t="s">
@@ -3756,7 +3764,7 @@
       <c r="E13" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F13" s="27">
+      <c r="F13" s="26">
         <v>26549502</v>
       </c>
       <c r="G13" s="8" t="s">
@@ -3923,18 +3931,18 @@
       <c r="BB13" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC13" s="28" t="s">
+      <c r="BC13" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD13" s="29">
+      <c r="BD13" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="14" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A14" s="6">
         <v>233</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="25" t="s">
         <v>67</v>
       </c>
       <c r="C14" s="7" t="s">
@@ -3946,7 +3954,7 @@
       <c r="E14" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F14" s="27">
+      <c r="F14" s="26">
         <v>90009500</v>
       </c>
       <c r="G14" s="2" t="s">
@@ -4114,18 +4122,18 @@
       <c r="BB14" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC14" s="28" t="s">
+      <c r="BC14" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD14" s="29">
+      <c r="BD14" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="15" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
         <v>928</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="30" t="s">
         <v>83</v>
       </c>
       <c r="C15" s="7" t="s">
@@ -4137,7 +4145,7 @@
       <c r="E15" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F15" s="27">
+      <c r="F15" s="26">
         <v>90018600</v>
       </c>
       <c r="G15" s="9" t="s">
@@ -4304,18 +4312,18 @@
       <c r="BB15" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC15" s="28" t="s">
+      <c r="BC15" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD15" s="29">
+      <c r="BD15" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="16" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A16" s="6">
         <v>926</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="25" t="s">
         <v>100</v>
       </c>
       <c r="C16" s="7" t="s">
@@ -4327,7 +4335,7 @@
       <c r="E16" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F16" s="27">
+      <c r="F16" s="26">
         <v>90016000</v>
       </c>
       <c r="G16" s="2" t="s">
@@ -4494,18 +4502,18 @@
       <c r="BB16" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC16" s="28" t="s">
+      <c r="BC16" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="BD16" s="29">
+      <c r="BD16" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="17" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A17" s="6">
         <v>981</v>
       </c>
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="25" t="s">
         <v>100</v>
       </c>
       <c r="C17" s="7" t="s">
@@ -4517,7 +4525,7 @@
       <c r="E17" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F17" s="27">
+      <c r="F17" s="26">
         <v>90016000</v>
       </c>
       <c r="G17" s="8" t="s">
@@ -4684,18 +4692,18 @@
       <c r="BB17" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="BC17" s="28" t="s">
+      <c r="BC17" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD17" s="29">
+      <c r="BD17" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="18" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A18" s="6">
         <v>120</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="25" t="s">
         <v>67</v>
       </c>
       <c r="C18" s="7" t="s">
@@ -4707,7 +4715,7 @@
       <c r="E18" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F18" s="27">
+      <c r="F18" s="26">
         <v>90009500</v>
       </c>
       <c r="G18" s="2" t="s">
@@ -4874,18 +4882,18 @@
       <c r="BB18" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC18" s="28" t="s">
+      <c r="BC18" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD18" s="29">
+      <c r="BD18" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="19" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A19" s="6">
         <v>915</v>
       </c>
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="25" t="s">
         <v>92</v>
       </c>
       <c r="C19" s="7" t="s">
@@ -4897,7 +4905,7 @@
       <c r="E19" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F19" s="27">
+      <c r="F19" s="26">
         <v>90012500</v>
       </c>
       <c r="G19" s="8" t="s">
@@ -5064,18 +5072,18 @@
       <c r="BB19" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC19" s="28" t="s">
+      <c r="BC19" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD19" s="29">
+      <c r="BD19" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="20" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A20" s="6">
         <v>917</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="25" t="s">
         <v>77</v>
       </c>
       <c r="C20" s="7" t="s">
@@ -5087,7 +5095,7 @@
       <c r="E20" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="F20" s="27">
+      <c r="F20" s="26">
         <v>90014400</v>
       </c>
       <c r="G20" s="2" t="s">
@@ -5254,18 +5262,18 @@
       <c r="BB20" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC20" s="28" t="s">
+      <c r="BC20" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD20" s="29">
+      <c r="BD20" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="21" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A21" s="6">
         <v>918</v>
       </c>
-      <c r="B21" s="30" t="s">
+      <c r="B21" s="29" t="s">
         <v>96</v>
       </c>
       <c r="C21" s="7" t="s">
@@ -5277,7 +5285,7 @@
       <c r="E21" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F21" s="27">
+      <c r="F21" s="26">
         <v>91017700</v>
       </c>
       <c r="G21" s="10" t="s">
@@ -5444,18 +5452,18 @@
       <c r="BB21" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC21" s="28" t="s">
+      <c r="BC21" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD21" s="29">
+      <c r="BD21" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="22" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A22" s="6">
         <v>925</v>
       </c>
-      <c r="B22" s="30" t="s">
+      <c r="B22" s="29" t="s">
         <v>83</v>
       </c>
       <c r="C22" s="7" t="s">
@@ -5467,7 +5475,7 @@
       <c r="E22" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F22" s="27">
+      <c r="F22" s="26">
         <v>90018600</v>
       </c>
       <c r="G22" s="8" t="s">
@@ -5634,18 +5642,18 @@
       <c r="BB22" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC22" s="28" t="s">
+      <c r="BC22" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD22" s="29">
+      <c r="BD22" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="23" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A23" s="6">
         <v>121</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="25" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="7" t="s">
@@ -5657,7 +5665,7 @@
       <c r="E23" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F23" s="27">
+      <c r="F23" s="26">
         <v>90009500</v>
       </c>
       <c r="G23" s="2" t="s">
@@ -5824,18 +5832,18 @@
       <c r="BB23" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC23" s="28" t="s">
+      <c r="BC23" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD23" s="29">
+      <c r="BD23" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="24" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A24" s="6">
         <v>912</v>
       </c>
-      <c r="B24" s="26" t="s">
+      <c r="B24" s="25" t="s">
         <v>83</v>
       </c>
       <c r="C24" s="7" t="s">
@@ -5847,7 +5855,7 @@
       <c r="E24" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F24" s="27">
+      <c r="F24" s="26">
         <v>90018600</v>
       </c>
       <c r="G24" s="2" t="s">
@@ -6014,18 +6022,18 @@
       <c r="BB24" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC24" s="28" t="s">
+      <c r="BC24" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD24" s="29">
+      <c r="BD24" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="25" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A25" s="6">
         <v>920</v>
       </c>
-      <c r="B25" s="30" t="s">
+      <c r="B25" s="29" t="s">
         <v>96</v>
       </c>
       <c r="C25" s="7" t="s">
@@ -6037,7 +6045,7 @@
       <c r="E25" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F25" s="27">
+      <c r="F25" s="26">
         <v>91017500</v>
       </c>
       <c r="G25" s="10" t="s">
@@ -6204,18 +6212,18 @@
       <c r="BB25" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC25" s="28" t="s">
+      <c r="BC25" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD25" s="29">
+      <c r="BD25" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="26" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A26" s="6">
         <v>921</v>
       </c>
-      <c r="B26" s="30" t="s">
+      <c r="B26" s="29" t="s">
         <v>77</v>
       </c>
       <c r="C26" s="7" t="s">
@@ -6227,7 +6235,7 @@
       <c r="E26" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F26" s="27">
+      <c r="F26" s="26">
         <v>90014400</v>
       </c>
       <c r="G26" s="8" t="s">
@@ -6394,18 +6402,18 @@
       <c r="BB26" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC26" s="28" t="s">
+      <c r="BC26" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD26" s="29">
+      <c r="BD26" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="27" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A27" s="6">
         <v>1001</v>
       </c>
-      <c r="B27" s="30" t="s">
+      <c r="B27" s="29" t="s">
         <v>83</v>
       </c>
       <c r="C27" s="7" t="s">
@@ -6417,7 +6425,7 @@
       <c r="E27" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="27">
+      <c r="F27" s="26">
         <v>90018600</v>
       </c>
       <c r="G27" s="8" t="s">
@@ -6584,18 +6592,18 @@
       <c r="BB27" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC27" s="28" t="s">
+      <c r="BC27" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="BD27" s="29">
+      <c r="BD27" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="28" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A28" s="6">
         <v>1063</v>
       </c>
-      <c r="B28" s="30" t="s">
+      <c r="B28" s="29" t="s">
         <v>77</v>
       </c>
       <c r="C28" s="7" t="s">
@@ -6607,7 +6615,7 @@
       <c r="E28" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F28" s="27">
+      <c r="F28" s="26">
         <v>90014400</v>
       </c>
       <c r="G28" s="8" t="s">
@@ -6774,18 +6782,18 @@
       <c r="BB28" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC28" s="28" t="s">
+      <c r="BC28" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="BD28" s="29">
+      <c r="BD28" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="29" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A29" s="6">
         <v>1005</v>
       </c>
-      <c r="B29" s="30" t="s">
+      <c r="B29" s="29" t="s">
         <v>107</v>
       </c>
       <c r="C29" s="7" t="s">
@@ -6797,7 +6805,7 @@
       <c r="E29" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F29" s="27">
+      <c r="F29" s="26">
         <v>9510600</v>
       </c>
       <c r="G29" s="8" t="s">
@@ -6964,18 +6972,18 @@
       <c r="BB29" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC29" s="28" t="s">
+      <c r="BC29" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD29" s="29">
+      <c r="BD29" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="30" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A30" s="6">
         <v>1006</v>
       </c>
-      <c r="B30" s="30" t="s">
+      <c r="B30" s="29" t="s">
         <v>110</v>
       </c>
       <c r="C30" s="7" t="s">
@@ -6987,7 +6995,7 @@
       <c r="E30" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F30" s="27">
+      <c r="F30" s="26">
         <v>90038200</v>
       </c>
       <c r="G30" s="8" t="s">
@@ -7154,18 +7162,18 @@
       <c r="BB30" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC30" s="28" t="s">
+      <c r="BC30" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD30" s="29">
+      <c r="BD30" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="31" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <v>1007</v>
       </c>
-      <c r="B31" s="30" t="s">
+      <c r="B31" s="29" t="s">
         <v>110</v>
       </c>
       <c r="C31" s="7" t="s">
@@ -7177,7 +7185,7 @@
       <c r="E31" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="F31" s="27">
+      <c r="F31" s="26">
         <v>900383</v>
       </c>
       <c r="G31" s="8" t="s">
@@ -7344,18 +7352,18 @@
       <c r="BB31" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC31" s="28" t="s">
+      <c r="BC31" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD31" s="29">
+      <c r="BD31" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="32" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A32" s="6">
         <v>1008</v>
       </c>
-      <c r="B32" s="30" t="s">
+      <c r="B32" s="29" t="s">
         <v>92</v>
       </c>
       <c r="C32" s="7" t="s">
@@ -7367,7 +7375,7 @@
       <c r="E32" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F32" s="27">
+      <c r="F32" s="26">
         <v>90016800</v>
       </c>
       <c r="G32" s="8" t="s">
@@ -7534,18 +7542,18 @@
       <c r="BB32" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC32" s="28" t="s">
+      <c r="BC32" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD32" s="29">
+      <c r="BD32" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="33" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A33" s="6">
         <v>1009</v>
       </c>
-      <c r="B33" s="30" t="s">
+      <c r="B33" s="29" t="s">
         <v>112</v>
       </c>
       <c r="C33" s="7" t="s">
@@ -7557,7 +7565,7 @@
       <c r="E33" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F33" s="27">
+      <c r="F33" s="26">
         <v>90016700</v>
       </c>
       <c r="G33" s="8" t="s">
@@ -7724,18 +7732,18 @@
       <c r="BB33" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC33" s="28" t="s">
+      <c r="BC33" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD33" s="29">
+      <c r="BD33" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="34" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A34" s="6">
         <v>1010</v>
       </c>
-      <c r="B34" s="30" t="s">
+      <c r="B34" s="29" t="s">
         <v>77</v>
       </c>
       <c r="C34" s="7" t="s">
@@ -7747,7 +7755,7 @@
       <c r="E34" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F34" s="27">
+      <c r="F34" s="26">
         <v>90017000</v>
       </c>
       <c r="G34" s="8" t="s">
@@ -7776,7 +7784,7 @@
         <v>14</v>
       </c>
       <c r="O34" s="4">
-        <f t="shared" ref="O34:O51" si="21">IF(I34="SFK Freight Forwarder",0,M34+N34-1)</f>
+        <f t="shared" ref="O34:O52" si="21">IF(I34="SFK Freight Forwarder",0,M34+N34-1)</f>
         <v>0</v>
       </c>
       <c r="P34" s="4">
@@ -7875,7 +7883,7 @@
         <v>3</v>
       </c>
       <c r="AQ34" s="4">
-        <f t="shared" ref="AQ34:AQ51" si="35">+AO34+AP34</f>
+        <f t="shared" ref="AQ34:AQ52" si="35">+AO34+AP34</f>
         <v>107</v>
       </c>
       <c r="AR34" s="4">
@@ -7914,18 +7922,18 @@
       <c r="BB34" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC34" s="28" t="s">
+      <c r="BC34" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD34" s="29">
+      <c r="BD34" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="35" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A35" s="6">
         <v>1012</v>
       </c>
-      <c r="B35" s="30" t="s">
+      <c r="B35" s="29" t="s">
         <v>83</v>
       </c>
       <c r="C35" s="7" t="s">
@@ -7937,7 +7945,7 @@
       <c r="E35" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F35" s="27">
+      <c r="F35" s="26">
         <v>90018000</v>
       </c>
       <c r="G35" s="8" t="s">
@@ -8104,18 +8112,18 @@
       <c r="BB35" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC35" s="28" t="s">
+      <c r="BC35" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD35" s="29">
+      <c r="BD35" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="36" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A36" s="6">
         <v>1034</v>
       </c>
-      <c r="B36" s="30" t="s">
+      <c r="B36" s="29" t="s">
         <v>96</v>
       </c>
       <c r="C36" s="7" t="s">
@@ -8127,7 +8135,7 @@
       <c r="E36" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F36" s="27">
+      <c r="F36" s="26">
         <v>91017300</v>
       </c>
       <c r="G36" s="8" t="s">
@@ -8294,18 +8302,18 @@
       <c r="BB36" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC36" s="28" t="s">
+      <c r="BC36" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD36" s="29">
+      <c r="BD36" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="37" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A37" s="6">
         <v>1037</v>
       </c>
-      <c r="B37" s="30" t="s">
+      <c r="B37" s="29" t="s">
         <v>100</v>
       </c>
       <c r="C37" s="7" t="s">
@@ -8317,7 +8325,7 @@
       <c r="E37" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F37" s="27">
+      <c r="F37" s="26">
         <v>90016000</v>
       </c>
       <c r="G37" s="8" t="s">
@@ -8484,18 +8492,18 @@
       <c r="BB37" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC37" s="28" t="s">
+      <c r="BC37" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD37" s="29">
+      <c r="BD37" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="38" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A38" s="6">
         <v>1040</v>
       </c>
-      <c r="B38" s="30" t="s">
+      <c r="B38" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C38" s="7" t="s">
@@ -8507,7 +8515,7 @@
       <c r="E38" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="F38" s="27">
+      <c r="F38" s="26">
         <v>26549502</v>
       </c>
       <c r="G38" s="8" t="s">
@@ -8674,18 +8682,18 @@
       <c r="BB38" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC38" s="28" t="s">
+      <c r="BC38" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD38" s="29">
+      <c r="BD38" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="39" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A39" s="6">
         <v>1029</v>
       </c>
-      <c r="B39" s="30" t="s">
+      <c r="B39" s="29" t="s">
         <v>92</v>
       </c>
       <c r="C39" s="7" t="s">
@@ -8697,7 +8705,7 @@
       <c r="E39" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="F39" s="27">
+      <c r="F39" s="26">
         <v>90012500</v>
       </c>
       <c r="G39" s="8" t="s">
@@ -8864,18 +8872,18 @@
       <c r="BB39" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC39" s="28" t="s">
+      <c r="BC39" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="BD39" s="29">
+      <c r="BD39" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="40" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A40" s="6">
         <v>1032</v>
       </c>
-      <c r="B40" s="30" t="s">
+      <c r="B40" s="29" t="s">
         <v>96</v>
       </c>
       <c r="C40" s="7" t="s">
@@ -8887,7 +8895,7 @@
       <c r="E40" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="F40" s="27">
+      <c r="F40" s="26">
         <v>91017500</v>
       </c>
       <c r="G40" s="8" t="s">
@@ -9054,18 +9062,18 @@
       <c r="BB40" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC40" s="28" t="s">
+      <c r="BC40" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="BD40" s="29">
+      <c r="BD40" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="41" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A41" s="6">
         <v>1033</v>
       </c>
-      <c r="B41" s="30" t="s">
+      <c r="B41" s="29" t="s">
         <v>86</v>
       </c>
       <c r="C41" s="7" t="s">
@@ -9077,7 +9085,7 @@
       <c r="E41" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="F41" s="27">
+      <c r="F41" s="26">
         <v>92000100</v>
       </c>
       <c r="G41" s="8" t="s">
@@ -9244,18 +9252,18 @@
       <c r="BB41" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC41" s="28" t="s">
+      <c r="BC41" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD41" s="29">
+      <c r="BD41" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="42" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A42" s="6">
         <v>904</v>
       </c>
-      <c r="B42" s="30" t="s">
+      <c r="B42" s="29" t="s">
         <v>77</v>
       </c>
       <c r="C42" s="7" t="s">
@@ -9267,7 +9275,7 @@
       <c r="E42" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F42" s="27">
+      <c r="F42" s="26">
         <v>90014400</v>
       </c>
       <c r="G42" s="10" t="s">
@@ -9434,18 +9442,18 @@
       <c r="BB42" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC42" s="28" t="s">
+      <c r="BC42" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD42" s="29">
+      <c r="BD42" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="43" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A43" s="6">
         <v>906</v>
       </c>
-      <c r="B43" s="30" t="s">
+      <c r="B43" s="29" t="s">
         <v>83</v>
       </c>
       <c r="C43" s="7" t="s">
@@ -9457,7 +9465,7 @@
       <c r="E43" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F43" s="27">
+      <c r="F43" s="26">
         <v>90018600</v>
       </c>
       <c r="G43" s="9" t="s">
@@ -9624,18 +9632,18 @@
       <c r="BB43" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC43" s="28" t="s">
+      <c r="BC43" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD43" s="29">
+      <c r="BD43" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="44" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A44" s="6">
         <v>924</v>
       </c>
-      <c r="B44" s="26" t="s">
+      <c r="B44" s="25" t="s">
         <v>92</v>
       </c>
       <c r="C44" s="7" t="s">
@@ -9647,7 +9655,7 @@
       <c r="E44" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="F44" s="27">
+      <c r="F44" s="26">
         <v>90012500</v>
       </c>
       <c r="G44" s="8" t="s">
@@ -9814,18 +9822,18 @@
       <c r="BB44" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC44" s="28" t="s">
+      <c r="BC44" s="27" t="s">
         <v>82</v>
       </c>
-      <c r="BD44" s="29">
+      <c r="BD44" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="45" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A45" s="6">
         <v>1014</v>
       </c>
-      <c r="B45" s="30" t="s">
+      <c r="B45" s="29" t="s">
         <v>107</v>
       </c>
       <c r="C45" s="7" t="s">
@@ -9837,7 +9845,7 @@
       <c r="E45" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F45" s="27">
+      <c r="F45" s="26">
         <v>9510600</v>
       </c>
       <c r="G45" s="8" t="s">
@@ -10004,18 +10012,18 @@
       <c r="BB45" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC45" s="28" t="s">
+      <c r="BC45" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD45" s="29">
+      <c r="BD45" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="46" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A46" s="6">
         <v>1015</v>
       </c>
-      <c r="B46" s="30" t="s">
+      <c r="B46" s="29" t="s">
         <v>83</v>
       </c>
       <c r="C46" s="7" t="s">
@@ -10027,7 +10035,7 @@
       <c r="E46" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F46" s="27">
+      <c r="F46" s="26">
         <v>90018000</v>
       </c>
       <c r="G46" s="8" t="s">
@@ -10194,18 +10202,18 @@
       <c r="BB46" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC46" s="28" t="s">
+      <c r="BC46" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD46" s="29">
+      <c r="BD46" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="47" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A47" s="6">
         <v>1036</v>
       </c>
-      <c r="B47" s="30" t="s">
+      <c r="B47" s="29" t="s">
         <v>96</v>
       </c>
       <c r="C47" s="7" t="s">
@@ -10217,7 +10225,7 @@
       <c r="E47" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="F47" s="27">
+      <c r="F47" s="26">
         <v>91017200</v>
       </c>
       <c r="G47" s="8" t="s">
@@ -10384,10 +10392,10 @@
       <c r="BB47" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC47" s="28" t="s">
+      <c r="BC47" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="BD47" s="29">
+      <c r="BD47" s="28">
         <v>46142</v>
       </c>
     </row>
@@ -10395,7 +10403,7 @@
       <c r="A48" s="6">
         <v>1084</v>
       </c>
-      <c r="B48" s="30" t="s">
+      <c r="B48" s="29" t="s">
         <v>83</v>
       </c>
       <c r="C48" s="7" t="s">
@@ -10407,7 +10415,7 @@
       <c r="E48" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F48" s="27">
+      <c r="F48" s="26">
         <v>90018600</v>
       </c>
       <c r="G48" s="8" t="s">
@@ -10574,18 +10582,18 @@
       <c r="BB48" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="BC48" s="28" t="s">
+      <c r="BC48" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="BD48" s="29">
+      <c r="BD48" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="49" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A49" s="6">
         <v>908</v>
       </c>
-      <c r="B49" s="31" t="s">
+      <c r="B49" s="30" t="s">
         <v>83</v>
       </c>
       <c r="C49" s="7" t="s">
@@ -10597,7 +10605,7 @@
       <c r="E49" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F49" s="27">
+      <c r="F49" s="26">
         <v>90018600</v>
       </c>
       <c r="G49" s="9" t="s">
@@ -10764,18 +10772,18 @@
       <c r="BB49" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC49" s="28" t="s">
+      <c r="BC49" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD49" s="29">
+      <c r="BD49" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="50" spans="1:56" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A50" s="6">
         <v>907</v>
       </c>
-      <c r="B50" s="31" t="s">
+      <c r="B50" s="30" t="s">
         <v>83</v>
       </c>
       <c r="C50" s="7" t="s">
@@ -10787,7 +10795,7 @@
       <c r="E50" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F50" s="27">
+      <c r="F50" s="26">
         <v>90018600</v>
       </c>
       <c r="G50" s="9" t="s">
@@ -10936,7 +10944,7 @@
       <c r="AV50" s="4">
         <v>17</v>
       </c>
-      <c r="AW50" s="33">
+      <c r="AW50" s="32">
         <f>+AE50+AG50+AI50</f>
         <v>37</v>
       </c>
@@ -10955,33 +10963,33 @@
       <c r="BB50" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="BC50" s="28" t="s">
+      <c r="BC50" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD50" s="29">
+      <c r="BD50" s="28">
         <v>46142</v>
       </c>
     </row>
-    <row r="51" spans="1:56" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="15">
+    <row r="51" spans="1:56" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="6">
         <v>1085</v>
       </c>
-      <c r="B51" s="31" t="s">
+      <c r="B51" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="C51" s="33" t="s">
+      <c r="C51" s="32" t="s">
         <v>84</v>
       </c>
       <c r="D51" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="E51" s="33" t="s">
+      <c r="E51" s="32" t="s">
         <v>103</v>
       </c>
-      <c r="F51" s="27">
+      <c r="F51" s="26">
         <v>90016500</v>
       </c>
-      <c r="G51" s="33" t="s">
+      <c r="G51" s="32" t="s">
         <v>156</v>
       </c>
       <c r="H51" s="3">
@@ -10993,7 +11001,7 @@
       <c r="J51" s="3">
         <v>29159</v>
       </c>
-      <c r="K51" s="33" t="s">
+      <c r="K51" s="32" t="s">
         <v>157</v>
       </c>
       <c r="L51" s="4">
@@ -11003,7 +11011,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="N51" s="33">
+      <c r="N51" s="32">
         <v>4</v>
       </c>
       <c r="O51" s="4">
@@ -11018,147 +11026,310 @@
         <f t="shared" si="23"/>
         <v>0</v>
       </c>
-      <c r="R51" s="33">
+      <c r="R51" s="32">
         <f t="shared" si="24"/>
         <v>13</v>
       </c>
-      <c r="S51" s="33">
+      <c r="S51" s="32">
         <v>4</v>
       </c>
-      <c r="T51" s="33">
+      <c r="T51" s="32">
         <f t="shared" si="25"/>
         <v>16</v>
       </c>
-      <c r="U51" s="33">
+      <c r="U51" s="32">
         <f t="shared" si="26"/>
         <v>17</v>
       </c>
-      <c r="V51" s="33">
-        <v>7</v>
-      </c>
-      <c r="W51" s="33">
+      <c r="V51" s="32">
+        <v>7</v>
+      </c>
+      <c r="W51" s="32">
         <f t="shared" si="27"/>
         <v>23</v>
       </c>
-      <c r="X51" s="33">
+      <c r="X51" s="32">
         <v>5</v>
       </c>
       <c r="Y51" s="4">
         <f t="shared" si="28"/>
         <v>26</v>
       </c>
-      <c r="Z51" s="33">
+      <c r="Z51" s="32">
         <v>29</v>
       </c>
       <c r="AA51" s="7">
         <f t="shared" si="29"/>
         <v>32</v>
       </c>
-      <c r="AB51" s="33">
+      <c r="AB51" s="32">
         <v>4</v>
       </c>
-      <c r="AC51" s="33"/>
-      <c r="AD51" s="33"/>
-      <c r="AE51" s="33">
+      <c r="AC51" s="32"/>
+      <c r="AD51" s="32"/>
+      <c r="AE51" s="32">
         <v>57</v>
       </c>
-      <c r="AF51" s="33">
+      <c r="AF51" s="32">
         <f t="shared" si="30"/>
         <v>88</v>
       </c>
-      <c r="AG51" s="33">
+      <c r="AG51" s="32">
         <v>3</v>
       </c>
-      <c r="AH51" s="33">
+      <c r="AH51" s="32">
         <f t="shared" si="31"/>
         <v>91</v>
       </c>
-      <c r="AI51" s="33">
-        <v>7</v>
-      </c>
-      <c r="AJ51" s="33">
+      <c r="AI51" s="32">
+        <v>7</v>
+      </c>
+      <c r="AJ51" s="32">
         <f t="shared" si="32"/>
         <v>98</v>
       </c>
-      <c r="AK51" s="33"/>
-      <c r="AL51" s="33">
+      <c r="AK51" s="32"/>
+      <c r="AL51" s="32">
         <v>3</v>
       </c>
-      <c r="AM51" s="33">
+      <c r="AM51" s="32">
         <f t="shared" si="33"/>
         <v>101</v>
       </c>
-      <c r="AN51" s="33">
+      <c r="AN51" s="32">
         <v>2</v>
       </c>
-      <c r="AO51" s="33">
+      <c r="AO51" s="32">
         <f t="shared" si="34"/>
         <v>103</v>
       </c>
-      <c r="AP51" s="33">
+      <c r="AP51" s="32">
         <v>2</v>
       </c>
-      <c r="AQ51" s="33">
+      <c r="AQ51" s="32">
         <f t="shared" si="35"/>
         <v>105</v>
       </c>
-      <c r="AR51" s="33">
+      <c r="AR51" s="32">
         <f t="shared" si="36"/>
         <v>112</v>
       </c>
-      <c r="AS51" s="33">
+      <c r="AS51" s="32">
         <f t="shared" si="37"/>
         <v>133</v>
       </c>
-      <c r="AT51" s="33">
+      <c r="AT51" s="32">
         <v>14</v>
       </c>
       <c r="AU51" s="4">
         <f t="shared" si="38"/>
         <v>19</v>
       </c>
-      <c r="AV51" s="33"/>
-      <c r="AW51" s="33">
+      <c r="AV51" s="32"/>
+      <c r="AW51" s="32">
         <f>+AE51+AG51+AI51</f>
         <v>67</v>
       </c>
-      <c r="AX51" s="33">
+      <c r="AX51" s="32">
         <f>+AQ51-R51+1</f>
         <v>93</v>
       </c>
-      <c r="AY51" s="33">
+      <c r="AY51" s="32">
         <f>+AQ51-L51+1</f>
         <v>101</v>
       </c>
-      <c r="AZ51" s="33"/>
-      <c r="BA51" s="33" t="s">
+      <c r="AZ51" s="32"/>
+      <c r="BA51" s="32" t="s">
         <v>152</v>
       </c>
-      <c r="BB51" s="33" t="s">
+      <c r="BB51" s="32" t="s">
         <v>150</v>
       </c>
-      <c r="BC51" s="28" t="s">
+      <c r="BC51" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="BD51" s="29">
+      <c r="BD51" s="28">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="52" spans="1:56" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B52" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="C52" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E52" s="32" t="s">
+        <v>159</v>
+      </c>
+      <c r="F52" s="26">
+        <v>91017700</v>
+      </c>
+      <c r="G52" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="H52" s="3">
+        <v>0</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="J52" s="3">
+        <v>29159</v>
+      </c>
+      <c r="K52" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="L52" s="4">
+        <v>7</v>
+      </c>
+      <c r="M52" s="4">
+        <v>0</v>
+      </c>
+      <c r="N52" s="32">
+        <v>0</v>
+      </c>
+      <c r="O52" s="4">
+        <v>0</v>
+      </c>
+      <c r="P52" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="4">
+        <v>0</v>
+      </c>
+      <c r="R52" s="32">
+        <v>0</v>
+      </c>
+      <c r="S52" s="32">
+        <v>0</v>
+      </c>
+      <c r="T52" s="32">
+        <v>0</v>
+      </c>
+      <c r="U52" s="32">
+        <v>7</v>
+      </c>
+      <c r="V52" s="32">
+        <v>7</v>
+      </c>
+      <c r="W52" s="32">
+        <v>14</v>
+      </c>
+      <c r="X52" s="32">
+        <v>1</v>
+      </c>
+      <c r="Y52" s="4">
+        <v>15</v>
+      </c>
+      <c r="Z52" s="32">
+        <v>18</v>
+      </c>
+      <c r="AA52" s="7">
+        <v>19</v>
+      </c>
+      <c r="AB52" s="32">
+        <v>4</v>
+      </c>
+      <c r="AC52" s="32"/>
+      <c r="AD52" s="32"/>
+      <c r="AE52" s="32">
+        <v>41</v>
+      </c>
+      <c r="AF52" s="32">
+        <f t="shared" ref="AF52" si="39">+AE52+AA52-1</f>
+        <v>59</v>
+      </c>
+      <c r="AG52" s="32">
+        <v>3</v>
+      </c>
+      <c r="AH52" s="32">
+        <f t="shared" ref="AH52" si="40">+AF52+AG52</f>
+        <v>62</v>
+      </c>
+      <c r="AI52" s="32">
+        <v>0</v>
+      </c>
+      <c r="AJ52" s="32">
+        <f t="shared" ref="AJ52" si="41">+AI52+AH52</f>
+        <v>62</v>
+      </c>
+      <c r="AK52" s="32"/>
+      <c r="AL52" s="32">
+        <v>3</v>
+      </c>
+      <c r="AM52" s="32">
+        <f t="shared" ref="AM52" si="42">+AJ52+AL52</f>
+        <v>65</v>
+      </c>
+      <c r="AN52" s="32">
+        <v>2</v>
+      </c>
+      <c r="AO52" s="32">
+        <f t="shared" ref="AO52" si="43">+AM52+AN52</f>
+        <v>67</v>
+      </c>
+      <c r="AP52" s="32">
+        <v>2</v>
+      </c>
+      <c r="AQ52" s="32">
+        <v>0</v>
+      </c>
+      <c r="AR52" s="32">
+        <v>0</v>
+      </c>
+      <c r="AS52" s="32">
+        <f t="shared" ref="AS52" si="44">+AR52+7+AT52</f>
+        <v>21</v>
+      </c>
+      <c r="AT52" s="32">
+        <v>14</v>
+      </c>
+      <c r="AU52" s="4">
+        <f t="shared" ref="AU52" si="45">+AA52-R52</f>
+        <v>19</v>
+      </c>
+      <c r="AV52" s="32"/>
+      <c r="AW52" s="32">
+        <f>+AE52+AG52+AI52</f>
+        <v>44</v>
+      </c>
+      <c r="AX52" s="32">
+        <f>+AQ52-R52+1</f>
+        <v>1</v>
+      </c>
+      <c r="AY52" s="32">
+        <f>+AU52+AW52+4</f>
+        <v>67</v>
+      </c>
+      <c r="AZ52" s="32"/>
+      <c r="BA52" s="32" t="s">
+        <v>152</v>
+      </c>
+      <c r="BB52" s="32" t="s">
+        <v>150</v>
+      </c>
+      <c r="BC52" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="BD52" s="28">
         <v>46143</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
-  <autoFilter ref="A1:BD51" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="MXVER"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <phoneticPr fontId="8" type="noConversion"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:E10 K2:K10 C14:E1048195 K14:K1048195" xr:uid="{833F6030-824F-4AAE-BA3C-131D886541AF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:E10 K2:K10 K14:K1048195 C14:E1048195" xr:uid="{833F6030-824F-4AAE-BA3C-131D886541AF}">
       <formula1>shippername</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:K51 H52:K1048195 C2:E1048195" xr:uid="{DD2A48DC-7068-4BD6-8A6F-E802386CE572}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:K52 C2:E1048195 H53:K1048195" xr:uid="{DD2A48DC-7068-4BD6-8A6F-E802386CE572}">
       <formula1>AILNname</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Please check information" error="This is not a known plant, please check the spelling or enter the information in the sheet &quot;Plant_ALIN&quot;" sqref="G2:G1048195" xr:uid="{D2D52A73-EC4B-4324-8BC4-BD77EF4C5461}">
@@ -11167,6 +11338,15 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;12&amp;K0000FF Internal Use</oddFooter>
+  </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9999a5d2-caa4-4f63-bace-dd6824b086db}" enabled="1" method="Standard" siteId="{de415ce7-227e-480f-88c9-c7dab50e161a}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Infimotion mas Jinrui VTTs
</commit_message>
<xml_diff>
--- a/VTT Tool/VTT DATA.xlsx
+++ b/VTT Tool/VTT DATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOJorge\Documents\Python projects\Horse Luis\VTT Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F679A5B8-B187-495D-BB0A-7ADF3FD61CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F412D0FA-01A6-4C61-83D3-2296F9AED2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
   </bookViews>
   <sheets>
     <sheet name="VTT actif" sheetId="1" r:id="rId1"/>
@@ -365,7 +365,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="163">
   <si>
     <t>Compte Consignee</t>
   </si>
@@ -844,13 +844,16 @@
     <t>O001</t>
   </si>
   <si>
-    <t>MAERSK</t>
-  </si>
-  <si>
     <t>DSV</t>
   </si>
   <si>
     <t>WUHAN JINRUI TECH</t>
+  </si>
+  <si>
+    <t>O002</t>
+  </si>
+  <si>
+    <t>EXPEDITORS</t>
   </si>
 </sst>
 </file>
@@ -861,7 +864,7 @@
     <numFmt numFmtId="164" formatCode="0000000000"/>
     <numFmt numFmtId="165" formatCode="00########"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -924,6 +927,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFF00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1025,7 +1036,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1125,6 +1136,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1467,7 +1481,8 @@
   <dimension ref="A1:BD52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="5" width="10.42578125" customWidth="1"/>
+    <col min="2" max="4" width="10.42578125" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.42578125" style="14" customWidth="1"/>
     <col min="7" max="7" width="15.42578125" customWidth="1"/>
     <col min="8" max="8" width="16" style="13" customWidth="1"/>
@@ -1934,7 +1949,7 @@
         <v>26</v>
       </c>
       <c r="Z3" s="7">
-        <f t="shared" ref="Z3:Z50" si="19">+Y3+X3-1</f>
+        <f t="shared" ref="Z3:Z51" si="19">+Y3+X3-1</f>
         <v>30</v>
       </c>
       <c r="AA3" s="7">
@@ -7792,18 +7807,18 @@
         <v>0</v>
       </c>
       <c r="Q34" s="4">
-        <f t="shared" ref="Q34:Q51" si="23">+IF(I34="SFK Freight Forwarder",0,O34+P34-1)</f>
+        <f t="shared" ref="Q34:Q52" si="23">+IF(I34="SFK Freight Forwarder",0,O34+P34-1)</f>
         <v>0</v>
       </c>
       <c r="R34" s="4">
-        <f t="shared" ref="R34:R51" si="24">9+N34</f>
+        <f t="shared" ref="R34:R52" si="24">9+N34</f>
         <v>23</v>
       </c>
       <c r="S34" s="4">
         <v>7</v>
       </c>
       <c r="T34" s="4">
-        <f t="shared" ref="T34:T51" si="25">+R34+S34-1</f>
+        <f t="shared" ref="T34:T52" si="25">+R34+S34-1</f>
         <v>29</v>
       </c>
       <c r="U34" s="4">
@@ -7814,7 +7829,7 @@
         <v>1</v>
       </c>
       <c r="W34" s="4">
-        <f t="shared" ref="W34:W51" si="27">+U34+V34-1</f>
+        <f t="shared" ref="W34:W52" si="27">+U34+V34-1</f>
         <v>30</v>
       </c>
       <c r="X34" s="4">
@@ -7829,7 +7844,7 @@
         <v>33</v>
       </c>
       <c r="AA34" s="7">
-        <f t="shared" ref="AA34:AA51" si="29">+Z34+AB34-1</f>
+        <f t="shared" ref="AA34:AA52" si="29">+Z34+AB34-1</f>
         <v>34</v>
       </c>
       <c r="AB34" s="4">
@@ -7887,7 +7902,7 @@
         <v>107</v>
       </c>
       <c r="AR34" s="4">
-        <f t="shared" ref="AR34:AR51" si="36">+AQ34+7</f>
+        <f t="shared" ref="AR34:AR52" si="36">+AQ34+7</f>
         <v>114</v>
       </c>
       <c r="AS34" s="4">
@@ -10971,8 +10986,8 @@
       </c>
     </row>
     <row r="51" spans="1:56" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="6">
-        <v>1085</v>
+      <c r="A51" s="6" t="s">
+        <v>158</v>
       </c>
       <c r="B51" s="30" t="s">
         <v>154</v>
@@ -10983,8 +10998,8 @@
       <c r="D51" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="E51" s="32" t="s">
-        <v>103</v>
+      <c r="E51" s="7" t="s">
+        <v>97</v>
       </c>
       <c r="F51" s="26">
         <v>90016500</v>
@@ -10996,7 +11011,7 @@
         <v>0</v>
       </c>
       <c r="I51" s="5" t="s">
-        <v>32</v>
+        <v>162</v>
       </c>
       <c r="J51" s="3">
         <v>29159</v>
@@ -11008,54 +11023,51 @@
         <v>5</v>
       </c>
       <c r="M51" s="4">
-        <f t="shared" si="20"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N51" s="32">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O51" s="4">
-        <f t="shared" si="21"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P51" s="4">
-        <f t="shared" si="22"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q51" s="4">
         <f t="shared" si="23"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="R51" s="32">
-        <f t="shared" si="24"/>
+        <v>9</v>
+      </c>
+      <c r="S51" s="32">
         <v>13</v>
-      </c>
-      <c r="S51" s="32">
-        <v>4</v>
       </c>
       <c r="T51" s="32">
         <f t="shared" si="25"/>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="U51" s="32">
         <f t="shared" si="26"/>
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="V51" s="32">
         <v>7</v>
       </c>
       <c r="W51" s="32">
         <f t="shared" si="27"/>
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="X51" s="32">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Y51" s="4">
         <f t="shared" si="28"/>
-        <v>26</v>
-      </c>
-      <c r="Z51" s="32">
+        <v>29</v>
+      </c>
+      <c r="Z51" s="7">
+        <f t="shared" si="19"/>
         <v>29</v>
       </c>
       <c r="AA51" s="7">
@@ -11123,7 +11135,7 @@
       </c>
       <c r="AU51" s="4">
         <f t="shared" si="38"/>
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="AV51" s="32"/>
       <c r="AW51" s="32">
@@ -11132,7 +11144,7 @@
       </c>
       <c r="AX51" s="32">
         <f>+AQ51-R51+1</f>
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="AY51" s="32">
         <f>+AQ51-L51+1</f>
@@ -11154,7 +11166,7 @@
     </row>
     <row r="52" spans="1:56" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B52" s="30" t="s">
         <v>96</v>
@@ -11166,7 +11178,7 @@
         <v>74</v>
       </c>
       <c r="E52" s="32" t="s">
-        <v>159</v>
+        <v>69</v>
       </c>
       <c r="F52" s="26">
         <v>91017700</v>
@@ -11178,61 +11190,67 @@
         <v>0</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J52" s="3">
         <v>29159</v>
       </c>
       <c r="K52" s="32" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L52" s="4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M52" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N52" s="32">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O52" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P52" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q52" s="4">
-        <v>0</v>
+        <f t="shared" si="23"/>
+        <v>12</v>
       </c>
       <c r="R52" s="32">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="S52" s="32">
-        <v>0</v>
-      </c>
-      <c r="T52" s="32">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="T52" s="34">
+        <f t="shared" si="25"/>
+        <v>21</v>
       </c>
       <c r="U52" s="32">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="V52" s="32">
         <v>7</v>
       </c>
       <c r="W52" s="32">
-        <v>14</v>
+        <f t="shared" si="27"/>
+        <v>22</v>
       </c>
       <c r="X52" s="32">
         <v>1</v>
       </c>
       <c r="Y52" s="4">
-        <v>15</v>
-      </c>
-      <c r="Z52" s="32">
-        <v>18</v>
+        <f t="shared" ref="Y52" si="39">+ROUNDDOWN(W52/7,0)*7+X52</f>
+        <v>22</v>
+      </c>
+      <c r="Z52" s="7">
+        <f t="shared" ref="Z52" si="40">+Y52+X52-1</f>
+        <v>22</v>
       </c>
       <c r="AA52" s="7">
-        <v>19</v>
+        <f t="shared" si="29"/>
+        <v>25</v>
       </c>
       <c r="AB52" s="32">
         <v>4</v>
@@ -11243,70 +11261,72 @@
         <v>41</v>
       </c>
       <c r="AF52" s="32">
-        <f t="shared" ref="AF52" si="39">+AE52+AA52-1</f>
-        <v>59</v>
+        <f t="shared" ref="AF52" si="41">+AE52+AA52-1</f>
+        <v>65</v>
       </c>
       <c r="AG52" s="32">
         <v>3</v>
       </c>
       <c r="AH52" s="32">
-        <f t="shared" ref="AH52" si="40">+AF52+AG52</f>
-        <v>62</v>
+        <f t="shared" ref="AH52" si="42">+AF52+AG52</f>
+        <v>68</v>
       </c>
       <c r="AI52" s="32">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AJ52" s="32">
-        <f t="shared" ref="AJ52" si="41">+AI52+AH52</f>
-        <v>62</v>
+        <f t="shared" ref="AJ52" si="43">+AI52+AH52</f>
+        <v>75</v>
       </c>
       <c r="AK52" s="32"/>
       <c r="AL52" s="32">
         <v>3</v>
       </c>
       <c r="AM52" s="32">
-        <f t="shared" ref="AM52" si="42">+AJ52+AL52</f>
-        <v>65</v>
+        <f t="shared" ref="AM52" si="44">+AJ52+AL52</f>
+        <v>78</v>
       </c>
       <c r="AN52" s="32">
         <v>2</v>
       </c>
       <c r="AO52" s="32">
-        <f t="shared" ref="AO52" si="43">+AM52+AN52</f>
-        <v>67</v>
+        <f t="shared" ref="AO52" si="45">+AM52+AN52</f>
+        <v>80</v>
       </c>
       <c r="AP52" s="32">
         <v>2</v>
       </c>
       <c r="AQ52" s="32">
-        <v>0</v>
+        <f t="shared" si="35"/>
+        <v>82</v>
       </c>
       <c r="AR52" s="32">
-        <v>0</v>
+        <f t="shared" si="36"/>
+        <v>89</v>
       </c>
       <c r="AS52" s="32">
-        <f t="shared" ref="AS52" si="44">+AR52+7+AT52</f>
-        <v>21</v>
+        <f t="shared" ref="AS52" si="46">+AR52+7+AT52</f>
+        <v>110</v>
       </c>
       <c r="AT52" s="32">
         <v>14</v>
       </c>
       <c r="AU52" s="4">
-        <f t="shared" ref="AU52" si="45">+AA52-R52</f>
-        <v>19</v>
+        <f t="shared" ref="AU52" si="47">+AA52-R52</f>
+        <v>16</v>
       </c>
       <c r="AV52" s="32"/>
       <c r="AW52" s="32">
         <f>+AE52+AG52+AI52</f>
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AX52" s="32">
         <f>+AQ52-R52+1</f>
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="AY52" s="32">
         <f>+AU52+AW52+4</f>
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="AZ52" s="32"/>
       <c r="BA52" s="32" t="s">
@@ -11329,7 +11349,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:E10 K2:K10 K14:K1048195 C14:E1048195" xr:uid="{833F6030-824F-4AAE-BA3C-131D886541AF}">
       <formula1>shippername</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:K52 C2:E1048195 H53:K1048195" xr:uid="{DD2A48DC-7068-4BD6-8A6F-E802386CE572}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:K52 H53:K1048195 C2:E1048195" xr:uid="{DD2A48DC-7068-4BD6-8A6F-E802386CE572}">
       <formula1>AILNname</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Please check information" error="This is not a known plant, please check the spelling or enter the information in the sheet &quot;Plant_ALIN&quot;" sqref="G2:G1048195" xr:uid="{D2D52A73-EC4B-4324-8BC4-BD77EF4C5461}">

</xml_diff>

<commit_message>
39 tt cn>pt infimotion
</commit_message>
<xml_diff>
--- a/VTT Tool/VTT DATA.xlsx
+++ b/VTT Tool/VTT DATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOJorge\Documents\Python projects\Horse Luis\VTT Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40930431-0DC3-44B2-9B50-B6E54B481E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE5EACD-C571-4E8A-9C6E-9380F8C04152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
   </bookViews>
   <sheets>
     <sheet name="VTT actif" sheetId="1" r:id="rId1"/>
@@ -43,6 +43,7 @@
   <authors>
     <author>ZHAO Tengda</author>
     <author>KERHOAS Delphine</author>
+    <author>OLMEDO Jorge</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{76836CDF-0CCC-4954-9A5F-D98726354FA2}">
@@ -360,6 +361,30 @@
         </r>
       </text>
     </comment>
+    <comment ref="AE51" authorId="2" shapeId="0" xr:uid="{03B2F475-038D-443C-85E7-A56E14FE222A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>OLMEDO Jorge:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+from 57 to 37 with new LSP</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -864,7 +889,7 @@
     <numFmt numFmtId="164" formatCode="0000000000"/>
     <numFmt numFmtId="165" formatCode="00########"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -939,8 +964,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1007,6 +1045,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1036,7 +1080,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1138,6 +1182,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -7792,18 +7839,18 @@
         <v>7</v>
       </c>
       <c r="M34" s="4">
-        <f t="shared" ref="M34:M51" si="20">+IF(I34="SFK Freight Forwarder",0,9)</f>
+        <f t="shared" ref="M34:M50" si="20">+IF(I34="SFK Freight Forwarder",0,9)</f>
         <v>0</v>
       </c>
       <c r="N34" s="4">
         <v>14</v>
       </c>
       <c r="O34" s="4">
-        <f t="shared" ref="O34:O52" si="21">IF(I34="SFK Freight Forwarder",0,M34+N34-1)</f>
+        <f t="shared" ref="O34:O50" si="21">IF(I34="SFK Freight Forwarder",0,M34+N34-1)</f>
         <v>0</v>
       </c>
       <c r="P34" s="4">
-        <f t="shared" ref="P34:P51" si="22">+IF(I34="SFK Freight Forwarder",0,5)</f>
+        <f t="shared" ref="P34:P50" si="22">+IF(I34="SFK Freight Forwarder",0,5)</f>
         <v>0</v>
       </c>
       <c r="Q34" s="4">
@@ -7811,7 +7858,7 @@
         <v>0</v>
       </c>
       <c r="R34" s="4">
-        <f t="shared" ref="R34:R52" si="24">9+N34</f>
+        <f t="shared" ref="R34:R50" si="24">9+N34</f>
         <v>23</v>
       </c>
       <c r="S34" s="4">
@@ -11079,26 +11126,26 @@
       </c>
       <c r="AC51" s="32"/>
       <c r="AD51" s="32"/>
-      <c r="AE51" s="32">
-        <v>57</v>
+      <c r="AE51" s="35">
+        <v>39</v>
       </c>
       <c r="AF51" s="32">
         <f t="shared" si="30"/>
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="AG51" s="32">
         <v>3</v>
       </c>
       <c r="AH51" s="32">
         <f t="shared" si="31"/>
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="AI51" s="32">
         <v>7</v>
       </c>
       <c r="AJ51" s="32">
         <f t="shared" si="32"/>
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="AK51" s="32"/>
       <c r="AL51" s="32">
@@ -11106,29 +11153,29 @@
       </c>
       <c r="AM51" s="32">
         <f t="shared" si="33"/>
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="AN51" s="32">
         <v>2</v>
       </c>
       <c r="AO51" s="32">
         <f t="shared" si="34"/>
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="AP51" s="32">
         <v>2</v>
       </c>
       <c r="AQ51" s="32">
         <f t="shared" si="35"/>
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="AR51" s="32">
         <f t="shared" si="36"/>
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="AS51" s="32">
         <f t="shared" si="37"/>
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="AT51" s="32">
         <v>14</v>
@@ -11140,15 +11187,15 @@
       <c r="AV51" s="32"/>
       <c r="AW51" s="32">
         <f>+AE51+AG51+AI51</f>
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="AX51" s="32">
         <f>+AQ51-R51+1</f>
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="AY51" s="32">
         <f>+AQ51-L51+1</f>
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="AZ51" s="32"/>
       <c r="BA51" s="32" t="s">

</xml_diff>

<commit_message>
tt infimotion a 41 days
</commit_message>
<xml_diff>
--- a/VTT Tool/VTT DATA.xlsx
+++ b/VTT Tool/VTT DATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOJorge\Documents\Python projects\Horse Luis\VTT Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D05D4012-0B3E-452D-A88C-57561EF47EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42016719-E28C-4D92-9897-093C7292BA97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-1340" windowWidth="19420" windowHeight="11500" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11295" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
   </bookViews>
   <sheets>
     <sheet name="VTT actif" sheetId="1" r:id="rId1"/>
@@ -1551,13 +1551,13 @@
     <col min="2" max="2" width="12.85546875" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="10.42578125" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" style="9" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="7" max="7" width="15.42578125" style="8" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="8" max="8" width="16" style="8" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="9" max="9" width="13.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="10" max="10" width="12.5703125" style="9" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="11" width="15.5703125" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="12" max="12" width="15.42578125" style="9" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="12.42578125" style="9" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="15.42578125" style="8" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="16" style="8" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="13.28515625" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="10" width="12.5703125" style="9" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="15.5703125" customWidth="1" outlineLevel="1"/>
+    <col min="12" max="12" width="15.42578125" style="9" customWidth="1"/>
     <col min="13" max="13" width="10.42578125" customWidth="1"/>
     <col min="14" max="14" width="14.5703125" customWidth="1"/>
     <col min="15" max="28" width="10.42578125" customWidth="1"/>
@@ -9514,25 +9514,25 @@
       <c r="AC46" s="23"/>
       <c r="AD46" s="23"/>
       <c r="AE46" s="33">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="AF46" s="23">
         <f t="shared" si="27"/>
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AG46" s="23">
         <v>3</v>
       </c>
       <c r="AH46" s="23">
         <f t="shared" si="28"/>
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AI46" s="23">
         <v>7</v>
       </c>
       <c r="AJ46" s="23">
         <f t="shared" si="29"/>
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AK46" s="23"/>
       <c r="AL46" s="23">
@@ -9540,29 +9540,29 @@
       </c>
       <c r="AM46" s="23">
         <f t="shared" si="30"/>
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AN46" s="23">
         <v>2</v>
       </c>
       <c r="AO46" s="23">
         <f t="shared" si="31"/>
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AP46" s="23">
         <v>2</v>
       </c>
       <c r="AQ46" s="23">
         <f t="shared" si="32"/>
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AR46" s="23">
         <f t="shared" si="33"/>
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AS46" s="23">
         <f t="shared" si="34"/>
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AT46" s="23">
         <v>14</v>

</xml_diff>

<commit_message>
actualizacion de ficheros de desgarga
</commit_message>
<xml_diff>
--- a/VTT Tool/VTT DATA.xlsx
+++ b/VTT Tool/VTT DATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOJorge\Documents\Python projects\Horse Luis\VTT Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42016719-E28C-4D92-9897-093C7292BA97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ED7C35A-062F-4CB2-9A65-A3844F7896EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11295" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
+    <workbookView xWindow="18860" yWindow="-890" windowWidth="21600" windowHeight="11300" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
   </bookViews>
   <sheets>
     <sheet name="VTT actif" sheetId="1" r:id="rId1"/>
@@ -1551,13 +1551,13 @@
     <col min="2" max="2" width="12.85546875" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="10.42578125" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" style="9" customWidth="1" outlineLevel="1"/>
-    <col min="7" max="7" width="15.42578125" style="8" customWidth="1" outlineLevel="1"/>
-    <col min="8" max="8" width="16" style="8" customWidth="1" outlineLevel="1"/>
-    <col min="9" max="9" width="13.28515625" customWidth="1" outlineLevel="1"/>
-    <col min="10" max="10" width="12.5703125" style="9" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="11" width="15.5703125" customWidth="1" outlineLevel="1"/>
-    <col min="12" max="12" width="15.42578125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" style="9" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="15.42578125" style="8" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="16" style="8" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="13.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="10" width="12.5703125" style="9" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="15.5703125" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="12" max="12" width="15.42578125" style="9" customWidth="1" collapsed="1"/>
     <col min="13" max="13" width="10.42578125" customWidth="1"/>
     <col min="14" max="14" width="14.5703125" customWidth="1"/>
     <col min="15" max="28" width="10.42578125" customWidth="1"/>
@@ -9456,35 +9456,34 @@
         <v>5</v>
       </c>
       <c r="M46" s="3">
-        <f t="shared" si="22"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N46" s="23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O46" s="3">
         <f t="shared" si="23"/>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P46" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q46" s="3">
         <f t="shared" si="24"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R46" s="23">
         <v>9</v>
       </c>
       <c r="S46" s="23">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="T46" s="23">
         <f t="shared" si="25"/>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="U46" s="23">
-        <f t="shared" si="6"/>
+        <f>+T46+2</f>
         <v>22</v>
       </c>
       <c r="V46" s="23">

</xml_diff>

<commit_message>
actualizacion de la UI
</commit_message>
<xml_diff>
--- a/VTT Tool/VTT DATA.xlsx
+++ b/VTT Tool/VTT DATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOJorge\Documents\Python projects\Horse Luis\VTT Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61087A30-B407-45A1-A38A-714E690EB8D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D324782C-1A39-4779-954A-12B55EB239D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
   </bookViews>
   <sheets>
     <sheet name="VTT actif" sheetId="1" r:id="rId1"/>
@@ -366,7 +366,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="173">
   <si>
     <t>Compte Consignee</t>
   </si>
@@ -791,9 +791,6 @@
     <t>WUHAN JINRUI TECH</t>
   </si>
   <si>
-    <t>O002</t>
-  </si>
-  <si>
     <t xml:space="preserve"> ILN/FF</t>
   </si>
   <si>
@@ -882,6 +879,12 @@
   </si>
   <si>
     <t>MAERSK</t>
+  </si>
+  <si>
+    <t>O010</t>
+  </si>
+  <si>
+    <t>Hapag-Lloyd</t>
   </si>
 </sst>
 </file>
@@ -1092,7 +1095,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1213,6 +1216,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1550,7 +1556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
-  <sheetPr codeName="Feuil4">
+  <sheetPr codeName="Feuil4" filterMode="1">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="A1:BF53"/>
@@ -1608,7 +1614,7 @@
         <v>1</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J1" s="12" t="s">
         <v>4</v>
@@ -1746,10 +1752,10 @@
         <v>63</v>
       </c>
       <c r="BF1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>60</v>
       </c>
@@ -1769,19 +1775,19 @@
         <v>90009500</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H2" s="2">
         <v>92000100</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J2" s="2">
         <v>92000100</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L2" s="3">
         <v>7</v>
@@ -1922,7 +1928,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="3" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>120</v>
       </c>
@@ -1942,7 +1948,7 @@
         <v>90009500</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H3" s="2">
         <v>2533780546</v>
@@ -2095,7 +2101,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="4" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>121</v>
       </c>
@@ -2115,7 +2121,7 @@
         <v>90009500</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H4" s="2">
         <v>2533780535</v>
@@ -2268,7 +2274,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="5" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>233</v>
       </c>
@@ -2288,7 +2294,7 @@
         <v>90009500</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H5" s="2">
         <v>91018400</v>
@@ -2441,7 +2447,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="6" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>416</v>
       </c>
@@ -2461,7 +2467,7 @@
         <v>90014400</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H6" s="2">
         <v>95207</v>
@@ -2614,7 +2620,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="7" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>752</v>
       </c>
@@ -2785,7 +2791,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="8" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>761</v>
       </c>
@@ -2955,7 +2961,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="9" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>888</v>
       </c>
@@ -3127,7 +3133,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="10" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>901</v>
       </c>
@@ -3147,7 +3153,7 @@
         <v>90012500</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H10" s="2">
         <v>95207</v>
@@ -3300,7 +3306,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="11" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>904</v>
       </c>
@@ -3314,13 +3320,13 @@
         <v>50</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F11" s="19">
         <v>90014400</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H11" s="2">
         <v>95436</v>
@@ -3473,7 +3479,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="12" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>906</v>
       </c>
@@ -3487,13 +3493,13 @@
         <v>62</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F12" s="19">
         <v>90018600</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H12" s="2">
         <v>95436</v>
@@ -3646,7 +3652,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="13" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>907</v>
       </c>
@@ -3666,7 +3672,7 @@
         <v>90018600</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H13" s="2">
         <v>95112</v>
@@ -3819,7 +3825,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="14" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>908</v>
       </c>
@@ -3839,7 +3845,7 @@
         <v>90018600</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H14" s="2">
         <v>28390</v>
@@ -3992,7 +3998,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="15" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>910</v>
       </c>
@@ -4006,25 +4012,25 @@
         <v>62</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F15" s="19">
         <v>90018600</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H15" s="2">
         <v>92000100</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J15" s="2">
         <v>92000100</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L15" s="3">
         <v>7</v>
@@ -4166,7 +4172,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="16" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>912</v>
       </c>
@@ -4186,7 +4192,7 @@
         <v>90018600</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H16" s="2">
         <v>2533780535</v>
@@ -4339,7 +4345,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="17" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>915</v>
       </c>
@@ -4359,7 +4365,7 @@
         <v>90012500</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H17" s="2">
         <v>2533780546</v>
@@ -4511,7 +4517,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="18" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>916</v>
       </c>
@@ -4531,7 +4537,7 @@
         <v>91017700</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H18" s="2">
         <v>95207</v>
@@ -4684,7 +4690,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="19" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>917</v>
       </c>
@@ -4704,7 +4710,7 @@
         <v>90014400</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H19" s="2">
         <v>2533780546</v>
@@ -4857,7 +4863,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="20" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>918</v>
       </c>
@@ -4877,7 +4883,7 @@
         <v>91017700</v>
       </c>
       <c r="G20" s="35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H20" s="2">
         <v>2533780546</v>
@@ -5030,7 +5036,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="21" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>920</v>
       </c>
@@ -5050,7 +5056,7 @@
         <v>91017500</v>
       </c>
       <c r="G21" s="35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H21" s="2">
         <v>2533780535</v>
@@ -5203,7 +5209,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="22" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>921</v>
       </c>
@@ -5223,7 +5229,7 @@
         <v>90014400</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H22" s="2">
         <v>2533780535</v>
@@ -5376,7 +5382,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="23" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>924</v>
       </c>
@@ -5396,7 +5402,7 @@
         <v>90012500</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H23" s="2">
         <v>92050300</v>
@@ -5549,7 +5555,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="24" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>925</v>
       </c>
@@ -5557,7 +5563,7 @@
         <v>67</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>62</v>
@@ -5569,7 +5575,7 @@
         <v>90018600</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H24" s="2">
         <v>2533780546</v>
@@ -5722,7 +5728,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="25" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>927</v>
       </c>
@@ -5742,7 +5748,7 @@
         <v>90014400</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H25" s="2">
         <v>26037000</v>
@@ -5895,7 +5901,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="26" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>928</v>
       </c>
@@ -5915,7 +5921,7 @@
         <v>90018600</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H26" s="2">
         <v>91018400</v>
@@ -6068,7 +6074,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="27" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>930</v>
       </c>
@@ -6088,7 +6094,7 @@
         <v>91017700</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H27" s="2">
         <v>26037000</v>
@@ -6240,7 +6246,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="28" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:51" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>931</v>
       </c>
@@ -6260,7 +6266,7 @@
         <v>90018600</v>
       </c>
       <c r="G28" s="36" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H28" s="2">
         <v>26037000</v>
@@ -6413,7 +6419,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="29" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>932</v>
       </c>
@@ -6433,7 +6439,7 @@
         <v>90012500</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H29" s="2">
         <v>26037000</v>
@@ -6586,7 +6592,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="30" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>1005</v>
       </c>
@@ -6758,7 +6764,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="31" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>1006</v>
       </c>
@@ -6930,7 +6936,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="32" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>1007</v>
       </c>
@@ -7104,7 +7110,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="33" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>1009</v>
       </c>
@@ -7118,7 +7124,7 @@
         <v>95</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F33" s="19">
         <v>90016700</v>
@@ -7276,7 +7282,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="34" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>1010</v>
       </c>
@@ -7448,7 +7454,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="35" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
         <v>1012</v>
       </c>
@@ -7621,7 +7627,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="36" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
         <v>1014</v>
       </c>
@@ -7793,7 +7799,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="37" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
         <v>1015</v>
       </c>
@@ -7965,7 +7971,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="38" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
         <v>1034</v>
       </c>
@@ -8137,7 +8143,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="39" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
         <v>1036</v>
       </c>
@@ -8309,7 +8315,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="40" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
         <v>1037</v>
       </c>
@@ -8481,7 +8487,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="41" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
         <v>1039</v>
       </c>
@@ -8501,7 +8507,7 @@
         <v>91017700</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H41" s="2">
         <v>222222</v>
@@ -8654,7 +8660,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="42" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
         <v>1040</v>
       </c>
@@ -8826,7 +8832,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="43" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
         <v>1045</v>
       </c>
@@ -8846,7 +8852,7 @@
         <v>90014400</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H43" s="2">
         <v>222222</v>
@@ -8999,7 +9005,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="44" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
         <v>1084</v>
       </c>
@@ -9013,13 +9019,13 @@
         <v>62</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F44" s="19">
         <v>90018600</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H44" s="2">
         <v>333333</v>
@@ -9172,7 +9178,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="45" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>138</v>
       </c>
@@ -9192,7 +9198,7 @@
         <v>90016500</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H45" s="2">
         <v>0</v>
@@ -9334,27 +9340,27 @@
         <v>46508</v>
       </c>
     </row>
-    <row r="46" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B46" s="38" t="s">
+        <v>171</v>
+      </c>
+      <c r="B46" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C46" s="39" t="s">
+      <c r="C46" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D46" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="E46" s="33" t="s">
-        <v>53</v>
+      <c r="D46" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E46" s="32" t="s">
+        <v>81</v>
       </c>
       <c r="F46" s="19">
-        <v>91017700</v>
-      </c>
-      <c r="G46" s="35" t="s">
-        <v>158</v>
+        <v>90016500</v>
+      </c>
+      <c r="G46" s="23" t="s">
+        <v>159</v>
       </c>
       <c r="H46" s="2">
         <v>0</v>
@@ -9366,126 +9372,122 @@
         <v>29159</v>
       </c>
       <c r="K46" s="23" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="L46" s="3">
         <v>5</v>
       </c>
       <c r="M46" s="3">
-        <f t="shared" si="35"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N46" s="23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O46" s="3">
-        <f t="shared" si="22"/>
-        <v>10</v>
+        <f t="shared" ref="O46" si="36">IF(I46="SFK Freight Forwarder",M46,M46+N46-1)</f>
+        <v>8</v>
       </c>
       <c r="P46" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q46" s="3">
-        <f t="shared" si="23"/>
-        <v>14</v>
+        <f t="shared" ref="Q46" si="37">+IF(I46="SFK Freight Forwarder",O46,O46+P46-1)</f>
+        <v>13</v>
       </c>
       <c r="R46" s="23">
         <v>9</v>
       </c>
       <c r="S46" s="23">
-        <v>13</v>
-      </c>
-      <c r="T46" s="25">
-        <f t="shared" si="24"/>
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="T46" s="23">
+        <f t="shared" ref="T46" si="38">+R46+S46-1</f>
+        <v>20</v>
       </c>
       <c r="U46" s="23">
-        <v>16</v>
+        <f>+T46+2</f>
+        <v>22</v>
       </c>
       <c r="V46" s="23">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W46" s="23">
-        <f t="shared" si="25"/>
-        <v>22</v>
+        <f t="shared" ref="W46" si="39">+U46+V46-1</f>
+        <v>26</v>
       </c>
       <c r="X46" s="23">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Y46" s="3">
-        <f t="shared" si="20"/>
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="Z46" s="6">
-        <f t="shared" ref="Z46:Z52" si="36">+Y46+X46-1</f>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="AA46" s="6">
-        <f t="shared" si="18"/>
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="AB46" s="23">
         <v>4</v>
       </c>
       <c r="AC46" s="23"/>
       <c r="AD46" s="23"/>
-      <c r="AE46" s="23">
-        <v>39</v>
+      <c r="AE46" s="33">
+        <v>34</v>
       </c>
       <c r="AF46" s="23">
-        <f t="shared" si="26"/>
-        <v>63</v>
+        <f t="shared" ref="AF46" si="40">+AE46+AA46-1</f>
+        <v>69</v>
       </c>
       <c r="AG46" s="23">
         <v>3</v>
       </c>
       <c r="AH46" s="23">
-        <f t="shared" si="27"/>
-        <v>66</v>
+        <f t="shared" ref="AH46" si="41">+AF46+AG46</f>
+        <v>72</v>
       </c>
       <c r="AI46" s="23">
         <v>7</v>
       </c>
       <c r="AJ46" s="23">
-        <f t="shared" si="28"/>
-        <v>73</v>
+        <f t="shared" ref="AJ46" si="42">+AI46+AH46</f>
+        <v>79</v>
       </c>
       <c r="AK46" s="23"/>
       <c r="AL46" s="23">
         <v>3</v>
       </c>
       <c r="AM46" s="23">
-        <f t="shared" si="29"/>
-        <v>76</v>
+        <f t="shared" ref="AM46" si="43">+AJ46+AL46</f>
+        <v>82</v>
       </c>
       <c r="AN46" s="23">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AO46" s="23">
-        <f t="shared" si="30"/>
-        <v>78</v>
+        <f>+AM46+AN46</f>
+        <v>87</v>
       </c>
       <c r="AP46" s="23">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AQ46" s="23">
-        <f t="shared" si="31"/>
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="AR46" s="23">
-        <f t="shared" si="32"/>
-        <v>87</v>
+        <f>+AQ46+4</f>
+        <v>96</v>
       </c>
       <c r="AS46" s="23">
-        <f t="shared" si="33"/>
-        <v>108</v>
+        <f t="shared" ref="AS46" si="44">+AR46+7+AT46</f>
+        <v>117</v>
       </c>
       <c r="AT46" s="23">
         <v>14</v>
       </c>
       <c r="AU46" s="3">
-        <f t="shared" si="34"/>
-        <v>16</v>
+        <f t="shared" ref="AU46" si="45">+AA46-R46</f>
+        <v>27</v>
       </c>
       <c r="AV46" s="23" t="s">
         <v>133</v>
@@ -9497,12 +9499,12 @@
         <v>56</v>
       </c>
       <c r="AY46" s="37">
-        <v>46143</v>
+        <v>46508</v>
       </c>
     </row>
-    <row r="47" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B47" s="39" t="s">
         <v>67</v>
@@ -9520,7 +9522,7 @@
         <v>90018600</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H47" s="2">
         <v>0</v>
@@ -9549,7 +9551,7 @@
         <v>22</v>
       </c>
       <c r="P47" s="3">
-        <f t="shared" ref="P47:P52" si="37">+IF(I47="SFK Freight Forwarder",0,5)</f>
+        <f t="shared" ref="P47:P52" si="46">+IF(I47="SFK Freight Forwarder",0,5)</f>
         <v>5</v>
       </c>
       <c r="Q47" s="3">
@@ -9557,7 +9559,7 @@
         <v>26</v>
       </c>
       <c r="R47" s="3">
-        <f t="shared" ref="R47:R52" si="38">9+N47</f>
+        <f t="shared" ref="R47:R52" si="47">9+N47</f>
         <v>23</v>
       </c>
       <c r="S47" s="3">
@@ -9568,7 +9570,7 @@
         <v>29</v>
       </c>
       <c r="U47" s="3">
-        <f t="shared" ref="U47:U52" si="39">+T47+1</f>
+        <f t="shared" ref="U47:U52" si="48">+T47+1</f>
         <v>30</v>
       </c>
       <c r="V47" s="3">
@@ -9586,7 +9588,7 @@
         <v>31</v>
       </c>
       <c r="Z47" s="6">
-        <f t="shared" si="36"/>
+        <f t="shared" ref="Z46:Z52" si="49">+Y47+X47-1</f>
         <v>33</v>
       </c>
       <c r="AA47" s="6">
@@ -9677,7 +9679,7 @@
     </row>
     <row r="48" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B48" s="39" t="s">
         <v>76</v>
@@ -9689,13 +9691,13 @@
         <v>77</v>
       </c>
       <c r="E48" s="38" t="s">
-        <v>85</v>
+        <v>172</v>
       </c>
       <c r="F48" s="19">
         <v>90012500</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H48" s="2">
         <v>0</v>
@@ -9707,7 +9709,7 @@
         <v>29159</v>
       </c>
       <c r="K48" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L48" s="3">
         <v>7</v>
@@ -9724,7 +9726,7 @@
         <v>22</v>
       </c>
       <c r="P48" s="3">
-        <f t="shared" si="37"/>
+        <f t="shared" si="46"/>
         <v>5</v>
       </c>
       <c r="Q48" s="3">
@@ -9732,7 +9734,7 @@
         <v>26</v>
       </c>
       <c r="R48" s="3">
-        <f t="shared" si="38"/>
+        <f t="shared" si="47"/>
         <v>23</v>
       </c>
       <c r="S48" s="3">
@@ -9743,7 +9745,7 @@
         <v>29</v>
       </c>
       <c r="U48" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="48"/>
         <v>30</v>
       </c>
       <c r="V48" s="3">
@@ -9754,19 +9756,16 @@
         <v>31</v>
       </c>
       <c r="X48" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y48" s="3">
-        <f t="shared" si="20"/>
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="Z48" s="6">
-        <f t="shared" si="36"/>
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="AA48" s="6">
-        <f t="shared" si="18"/>
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="AB48" s="3">
         <v>1</v>
@@ -9778,25 +9777,25 @@
         <v>10</v>
       </c>
       <c r="AE48" s="3">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="AF48" s="3">
         <f t="shared" si="26"/>
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="AG48" s="6">
         <v>3</v>
       </c>
       <c r="AH48" s="6">
         <f t="shared" si="27"/>
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="AI48" s="3">
         <v>0</v>
       </c>
       <c r="AJ48" s="3">
         <f t="shared" si="28"/>
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="AK48" s="3" t="s">
         <v>60</v>
@@ -9806,36 +9805,36 @@
       </c>
       <c r="AM48" s="3">
         <f t="shared" si="29"/>
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="AN48" s="3">
         <v>7</v>
       </c>
       <c r="AO48" s="3">
         <f t="shared" si="30"/>
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="AP48" s="3">
         <v>5</v>
       </c>
       <c r="AQ48" s="3">
         <f t="shared" si="31"/>
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="AR48" s="3">
         <f t="shared" si="32"/>
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="AS48" s="3">
         <f t="shared" si="33"/>
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="AT48" s="3">
         <v>0</v>
       </c>
       <c r="AU48" s="3">
         <f t="shared" si="34"/>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="AV48" s="3" t="s">
         <v>133</v>
@@ -9847,12 +9846,12 @@
         <v>88</v>
       </c>
       <c r="AY48" s="37">
-        <v>46142</v>
+        <v>46507</v>
       </c>
     </row>
-    <row r="49" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B49" s="39" t="s">
         <v>80</v>
@@ -9867,10 +9866,10 @@
         <v>53</v>
       </c>
       <c r="F49" s="19">
-        <v>91017500</v>
+        <v>90016500</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H49" s="2">
         <v>0</v>
@@ -9882,7 +9881,7 @@
         <v>29159</v>
       </c>
       <c r="K49" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L49" s="3">
         <v>7</v>
@@ -9899,7 +9898,7 @@
         <v>22</v>
       </c>
       <c r="P49" s="3">
-        <f t="shared" si="37"/>
+        <f t="shared" si="46"/>
         <v>5</v>
       </c>
       <c r="Q49" s="3">
@@ -9907,7 +9906,7 @@
         <v>26</v>
       </c>
       <c r="R49" s="3">
-        <f t="shared" si="38"/>
+        <f t="shared" si="47"/>
         <v>23</v>
       </c>
       <c r="S49" s="3">
@@ -9918,7 +9917,7 @@
         <v>29</v>
       </c>
       <c r="U49" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="48"/>
         <v>30</v>
       </c>
       <c r="V49" s="3">
@@ -9932,16 +9931,14 @@
         <v>2</v>
       </c>
       <c r="Y49" s="3">
-        <f t="shared" si="20"/>
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Z49" s="6">
-        <f t="shared" si="36"/>
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="AA49" s="6">
         <f t="shared" si="18"/>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="AB49" s="3">
         <v>6</v>
@@ -9953,25 +9950,25 @@
         <v>7</v>
       </c>
       <c r="AE49" s="3">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="AF49" s="3">
         <f t="shared" si="26"/>
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AG49" s="6">
         <v>3</v>
       </c>
       <c r="AH49" s="6">
         <f t="shared" si="27"/>
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="AI49" s="3">
         <v>0</v>
       </c>
       <c r="AJ49" s="3">
         <f t="shared" si="28"/>
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="AK49" s="3" t="s">
         <v>60</v>
@@ -9981,36 +9978,36 @@
       </c>
       <c r="AM49" s="3">
         <f t="shared" si="29"/>
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="AN49" s="3">
         <v>1</v>
       </c>
       <c r="AO49" s="3">
         <f t="shared" si="30"/>
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AP49" s="3">
         <v>3</v>
       </c>
       <c r="AQ49" s="3">
         <f t="shared" si="31"/>
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="AR49" s="3">
         <f t="shared" si="32"/>
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AS49" s="3">
         <f t="shared" si="33"/>
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="AT49" s="3">
         <v>0</v>
       </c>
       <c r="AU49" s="3">
         <f t="shared" si="34"/>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AV49" s="3" t="s">
         <v>133</v>
@@ -10021,13 +10018,13 @@
       <c r="AX49" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="AY49" s="37">
-        <v>46142</v>
+      <c r="AY49" s="41">
+        <v>46507</v>
       </c>
     </row>
-    <row r="50" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B50" s="39" t="s">
         <v>70</v>
@@ -10057,7 +10054,7 @@
         <v>29159</v>
       </c>
       <c r="K50" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L50" s="3">
         <v>7</v>
@@ -10074,7 +10071,7 @@
         <v>22</v>
       </c>
       <c r="P50" s="3">
-        <f t="shared" si="37"/>
+        <f t="shared" si="46"/>
         <v>5</v>
       </c>
       <c r="Q50" s="3">
@@ -10082,7 +10079,7 @@
         <v>26</v>
       </c>
       <c r="R50" s="3">
-        <f t="shared" si="38"/>
+        <f t="shared" si="47"/>
         <v>23</v>
       </c>
       <c r="S50" s="3">
@@ -10093,7 +10090,7 @@
         <v>29</v>
       </c>
       <c r="U50" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="48"/>
         <v>30</v>
       </c>
       <c r="V50" s="3">
@@ -10111,7 +10108,7 @@
         <v>30</v>
       </c>
       <c r="Z50" s="6">
-        <f t="shared" si="36"/>
+        <f t="shared" si="49"/>
         <v>31</v>
       </c>
       <c r="AA50" s="6">
@@ -10200,9 +10197,9 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="51" spans="1:51" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:51" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B51" s="39" t="s">
         <v>61</v>
@@ -10220,7 +10217,7 @@
         <v>90014400</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H51" s="2">
         <v>0</v>
@@ -10249,7 +10246,7 @@
         <v>22</v>
       </c>
       <c r="P51" s="3">
-        <f t="shared" si="37"/>
+        <f t="shared" si="46"/>
         <v>5</v>
       </c>
       <c r="Q51" s="3">
@@ -10257,7 +10254,7 @@
         <v>26</v>
       </c>
       <c r="R51" s="3">
-        <f t="shared" si="38"/>
+        <f t="shared" si="47"/>
         <v>23</v>
       </c>
       <c r="S51" s="3">
@@ -10268,7 +10265,7 @@
         <v>29</v>
       </c>
       <c r="U51" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="48"/>
         <v>30</v>
       </c>
       <c r="V51" s="3">
@@ -10286,7 +10283,7 @@
         <v>31</v>
       </c>
       <c r="Z51" s="6">
-        <f t="shared" si="36"/>
+        <f t="shared" si="49"/>
         <v>33</v>
       </c>
       <c r="AA51" s="6">
@@ -10375,9 +10372,9 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="52" spans="1:51" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:51" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B52" s="38" t="s">
         <v>83</v>
@@ -10389,7 +10386,7 @@
         <v>86</v>
       </c>
       <c r="E52" s="38" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="F52" s="19">
         <v>90016000</v>
@@ -10407,7 +10404,7 @@
         <v>5915200</v>
       </c>
       <c r="K52" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L52" s="3">
         <v>7</v>
@@ -10424,7 +10421,7 @@
         <v>15</v>
       </c>
       <c r="P52" s="3">
-        <f t="shared" si="37"/>
+        <f t="shared" si="46"/>
         <v>5</v>
       </c>
       <c r="Q52" s="3">
@@ -10432,7 +10429,7 @@
         <v>19</v>
       </c>
       <c r="R52" s="3">
-        <f t="shared" si="38"/>
+        <f t="shared" si="47"/>
         <v>16</v>
       </c>
       <c r="S52" s="3">
@@ -10443,7 +10440,7 @@
         <v>18</v>
       </c>
       <c r="U52" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="48"/>
         <v>19</v>
       </c>
       <c r="V52" s="3">
@@ -10461,12 +10458,11 @@
         <v>23</v>
       </c>
       <c r="Z52" s="6">
-        <f t="shared" si="36"/>
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AA52" s="6">
         <f t="shared" si="18"/>
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="AB52" s="3">
         <v>3</v>
@@ -10478,25 +10474,25 @@
         <v>5</v>
       </c>
       <c r="AE52" s="3">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="AF52" s="3">
         <f t="shared" si="26"/>
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="AG52" s="6">
         <v>3</v>
       </c>
       <c r="AH52" s="6">
         <f t="shared" si="27"/>
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="AI52" s="3">
         <v>7</v>
       </c>
       <c r="AJ52" s="3">
         <f t="shared" si="28"/>
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="AK52" s="3">
         <v>0</v>
@@ -10506,36 +10502,36 @@
       </c>
       <c r="AM52" s="3">
         <f t="shared" si="29"/>
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AN52" s="3">
         <v>2</v>
       </c>
       <c r="AO52" s="3">
         <f t="shared" si="30"/>
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AP52" s="3">
         <v>0</v>
       </c>
       <c r="AQ52" s="3">
         <f t="shared" si="31"/>
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AR52" s="3">
         <f t="shared" si="32"/>
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="AS52" s="3">
         <f t="shared" si="33"/>
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="AT52" s="3">
         <v>0</v>
       </c>
       <c r="AU52" s="3">
         <f t="shared" si="34"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AV52" s="3" t="s">
         <v>133</v>
@@ -10546,13 +10542,13 @@
       <c r="AX52" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="AY52" s="37">
-        <v>46142</v>
+      <c r="AY52" s="41">
+        <v>46507</v>
       </c>
     </row>
-    <row r="53" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B53" s="38" t="s">
         <v>61</v>
@@ -10570,7 +10566,7 @@
         <v>90014400</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H53" s="2">
         <v>0</v>
@@ -10588,21 +10584,21 @@
         <v>5</v>
       </c>
       <c r="M53" s="3">
-        <f t="shared" ref="M53" si="40">+IF(I53="SFK Freight Forwarder",L53,9)</f>
+        <f t="shared" ref="M53" si="50">+IF(I53="SFK Freight Forwarder",L53,9)</f>
         <v>9</v>
       </c>
       <c r="N53" s="23">
         <v>2</v>
       </c>
       <c r="O53" s="3">
-        <f t="shared" ref="O53" si="41">IF(I53="SFK Freight Forwarder",M53,M53+N53-1)</f>
+        <f t="shared" ref="O53" si="51">IF(I53="SFK Freight Forwarder",M53,M53+N53-1)</f>
         <v>10</v>
       </c>
       <c r="P53" s="3">
         <v>5</v>
       </c>
       <c r="Q53" s="3">
-        <f t="shared" ref="Q53" si="42">+IF(I53="SFK Freight Forwarder",O53,O53+P53-1)</f>
+        <f t="shared" ref="Q53" si="52">+IF(I53="SFK Freight Forwarder",O53,O53+P53-1)</f>
         <v>14</v>
       </c>
       <c r="R53" s="23">
@@ -10621,7 +10617,7 @@
         <v>4</v>
       </c>
       <c r="W53" s="23">
-        <f t="shared" ref="W53" si="43">+U53+V53-1</f>
+        <f t="shared" ref="W53" si="53">+U53+V53-1</f>
         <v>18</v>
       </c>
       <c r="X53" s="23">
@@ -10634,7 +10630,7 @@
         <v>19</v>
       </c>
       <c r="AA53" s="6">
-        <f t="shared" ref="AA53" si="44">+Z53+AB53-1</f>
+        <f t="shared" ref="AA53" si="54">+Z53+AB53-1</f>
         <v>22</v>
       </c>
       <c r="AB53" s="23">
@@ -10646,21 +10642,21 @@
         <v>46</v>
       </c>
       <c r="AF53" s="23">
-        <f t="shared" ref="AF53" si="45">+AE53+AA53-1</f>
+        <f t="shared" ref="AF53" si="55">+AE53+AA53-1</f>
         <v>67</v>
       </c>
       <c r="AG53" s="23">
         <v>3</v>
       </c>
       <c r="AH53" s="23">
-        <f t="shared" ref="AH53" si="46">+AF53+AG53</f>
+        <f t="shared" ref="AH53" si="56">+AF53+AG53</f>
         <v>70</v>
       </c>
       <c r="AI53" s="23">
         <v>7</v>
       </c>
       <c r="AJ53" s="23">
-        <f t="shared" ref="AJ53" si="47">+AI53+AH53</f>
+        <f t="shared" ref="AJ53" si="57">+AI53+AH53</f>
         <v>77</v>
       </c>
       <c r="AK53" s="23"/>
@@ -10668,36 +10664,36 @@
         <v>3</v>
       </c>
       <c r="AM53" s="23">
-        <f t="shared" ref="AM53" si="48">+AJ53+AL53</f>
+        <f t="shared" ref="AM53" si="58">+AJ53+AL53</f>
         <v>80</v>
       </c>
       <c r="AN53" s="23">
         <v>2</v>
       </c>
       <c r="AO53" s="23">
-        <f t="shared" ref="AO53" si="49">+AM53+AN53</f>
+        <f t="shared" ref="AO53" si="59">+AM53+AN53</f>
         <v>82</v>
       </c>
       <c r="AP53" s="23">
         <v>2</v>
       </c>
       <c r="AQ53" s="23">
-        <f t="shared" ref="AQ53" si="50">+AO53+AP53</f>
+        <f t="shared" ref="AQ53" si="60">+AO53+AP53</f>
         <v>84</v>
       </c>
       <c r="AR53" s="23">
-        <f t="shared" ref="AR53" si="51">+AQ53+7</f>
+        <f t="shared" ref="AR53" si="61">+AQ53+7</f>
         <v>91</v>
       </c>
       <c r="AS53" s="23">
-        <f t="shared" ref="AS53" si="52">+AR53+7+AT53</f>
+        <f t="shared" ref="AS53" si="62">+AR53+7+AT53</f>
         <v>112</v>
       </c>
       <c r="AT53" s="23">
         <v>14</v>
       </c>
       <c r="AU53" s="3">
-        <f t="shared" ref="AU53" si="53">+AA53-R53</f>
+        <f t="shared" ref="AU53" si="63">+AA53-R53</f>
         <v>22</v>
       </c>
       <c r="AV53" s="23" t="s">
@@ -10715,13 +10711,24 @@
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
-  <autoFilter ref="A1:AY53" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}"/>
+  <autoFilter ref="A1:AY53" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="O004"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="2">
+      <filters>
+        <filter val="JPYOK"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="8" type="noConversion"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:E12 K2:K12 K16:K1048195 C16:E1048195" xr:uid="{833F6030-824F-4AAE-BA3C-131D886541AF}">
       <formula1>shippername</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J10 H54:K1048195 C2:E1048195 I2:I53 J12:J53 K2:K53" xr:uid="{DD2A48DC-7068-4BD6-8A6F-E802386CE572}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J10 H54:K1048195 K2:K53 J12:J53 I2:I53 C2:E1048195" xr:uid="{DD2A48DC-7068-4BD6-8A6F-E802386CE572}">
       <formula1>AILNname</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Please check information" error="This is not a known plant, please check the spelling or enter the information in the sheet &quot;Plant_ALIN&quot;" sqref="G2:G1048195" xr:uid="{D2D52A73-EC4B-4324-8BC4-BD77EF4C5461}">
@@ -10744,35 +10751,35 @@
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C2" t="s">
         <v>162</v>
-      </c>
-      <c r="C2" t="s">
-        <v>163</v>
       </c>
       <c r="D2" t="s">
         <v>133</v>
       </c>
       <c r="E2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
+        <v>164</v>
+      </c>
+      <c r="C3" t="s">
         <v>165</v>
-      </c>
-      <c r="C3" t="s">
-        <v>166</v>
       </c>
       <c r="D3" t="s">
         <v>133</v>
       </c>
       <c r="E3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualizacion de las vista vtt
</commit_message>
<xml_diff>
--- a/VTT Tool/VTT DATA.xlsx
+++ b/VTT Tool/VTT DATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOJorge\Documents\Python projects\Horse Luis\VTT Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D324782C-1A39-4779-954A-12B55EB239D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B982F05A-18E9-4BA7-92FB-206CDAEABDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
   </bookViews>
   <sheets>
     <sheet name="VTT actif" sheetId="1" r:id="rId1"/>
@@ -1556,7 +1556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
-  <sheetPr codeName="Feuil4" filterMode="1">
+  <sheetPr codeName="Feuil4">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="A1:BF53"/>
@@ -1755,7 +1755,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>60</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="3" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>120</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="4" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>121</v>
       </c>
@@ -2274,7 +2274,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="5" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>233</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="6" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>416</v>
       </c>
@@ -2620,7 +2620,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="7" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>752</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="8" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>761</v>
       </c>
@@ -2961,7 +2961,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="9" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>888</v>
       </c>
@@ -3133,7 +3133,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="10" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>901</v>
       </c>
@@ -3306,7 +3306,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="11" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>904</v>
       </c>
@@ -3479,7 +3479,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="12" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>906</v>
       </c>
@@ -3652,7 +3652,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="13" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>907</v>
       </c>
@@ -3825,7 +3825,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="14" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>908</v>
       </c>
@@ -3998,7 +3998,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="15" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>910</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="16" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>912</v>
       </c>
@@ -4345,7 +4345,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="17" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>915</v>
       </c>
@@ -4517,7 +4517,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="18" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>916</v>
       </c>
@@ -4690,7 +4690,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="19" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>917</v>
       </c>
@@ -4863,7 +4863,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="20" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>918</v>
       </c>
@@ -5036,7 +5036,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="21" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>920</v>
       </c>
@@ -5209,7 +5209,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="22" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>921</v>
       </c>
@@ -5382,7 +5382,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="23" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>924</v>
       </c>
@@ -5555,7 +5555,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="24" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>925</v>
       </c>
@@ -5728,7 +5728,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="25" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>927</v>
       </c>
@@ -5901,7 +5901,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="26" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>928</v>
       </c>
@@ -6074,7 +6074,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="27" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>930</v>
       </c>
@@ -6246,7 +6246,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="28" spans="1:51" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>931</v>
       </c>
@@ -6419,7 +6419,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="29" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>932</v>
       </c>
@@ -6592,7 +6592,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="30" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>1005</v>
       </c>
@@ -6764,7 +6764,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="31" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>1006</v>
       </c>
@@ -6936,7 +6936,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="32" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>1007</v>
       </c>
@@ -7110,7 +7110,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="33" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>1009</v>
       </c>
@@ -7282,7 +7282,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="34" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>1010</v>
       </c>
@@ -7454,7 +7454,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="35" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
         <v>1012</v>
       </c>
@@ -7627,7 +7627,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="36" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
         <v>1014</v>
       </c>
@@ -7799,7 +7799,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="37" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
         <v>1015</v>
       </c>
@@ -7971,7 +7971,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="38" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
         <v>1034</v>
       </c>
@@ -8143,7 +8143,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="39" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
         <v>1036</v>
       </c>
@@ -8315,7 +8315,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="40" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
         <v>1037</v>
       </c>
@@ -8487,7 +8487,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="41" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
         <v>1039</v>
       </c>
@@ -8660,7 +8660,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="42" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
         <v>1040</v>
       </c>
@@ -8832,7 +8832,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="43" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
         <v>1045</v>
       </c>
@@ -9005,7 +9005,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="44" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
         <v>1084</v>
       </c>
@@ -9178,7 +9178,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="45" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>138</v>
       </c>
@@ -9340,7 +9340,7 @@
         <v>46508</v>
       </c>
     </row>
-    <row r="46" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>171</v>
       </c>
@@ -9502,7 +9502,7 @@
         <v>46508</v>
       </c>
     </row>
-    <row r="47" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>143</v>
       </c>
@@ -9849,7 +9849,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="49" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>145</v>
       </c>
@@ -10022,7 +10022,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="50" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>146</v>
       </c>
@@ -10197,7 +10197,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="51" spans="1:51" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:51" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>147</v>
       </c>
@@ -10372,7 +10372,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="52" spans="1:51" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:51" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>152</v>
       </c>
@@ -10546,7 +10546,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="53" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>168</v>
       </c>
@@ -10559,7 +10559,7 @@
       <c r="D53" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E53" s="33" t="s">
+      <c r="E53" s="38" t="s">
         <v>81</v>
       </c>
       <c r="F53" s="19">
@@ -10711,18 +10711,7 @@
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
-  <autoFilter ref="A1:AY53" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="O004"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="2">
-      <filters>
-        <filter val="JPYOK"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:AY53" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}"/>
   <phoneticPr fontId="8" type="noConversion"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:E12 K2:K12 K16:K1048195 C16:E1048195" xr:uid="{833F6030-824F-4AAE-BA3C-131D886541AF}">

</xml_diff>

<commit_message>
actualizacion de filtros y vista
</commit_message>
<xml_diff>
--- a/VTT Tool/VTT DATA.xlsx
+++ b/VTT Tool/VTT DATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOJorge\Documents\Python projects\Horse Luis\VTT Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B982F05A-18E9-4BA7-92FB-206CDAEABDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0FB66B7-7CC1-4730-AC7F-497F91A353D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
   </bookViews>
   <sheets>
     <sheet name="VTT actif" sheetId="1" r:id="rId1"/>
@@ -881,10 +881,10 @@
     <t>MAERSK</t>
   </si>
   <si>
-    <t>O010</t>
-  </si>
-  <si>
     <t>Hapag-Lloyd</t>
+  </si>
+  <si>
+    <t>O002</t>
   </si>
 </sst>
 </file>
@@ -1095,7 +1095,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1216,9 +1216,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1556,39 +1553,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
-  <sheetPr codeName="Feuil4">
+  <sheetPr codeName="Feuil4" filterMode="1">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="A1:BF53"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.42578125" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.453125" defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.42578125" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" style="9" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="7" max="7" width="15.42578125" style="8" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="1" max="1" width="9.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.453125" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.453125" style="9" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="15.453125" style="8" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="8" max="8" width="16" style="8" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="9" max="9" width="13.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="10" max="10" width="12.5703125" style="9" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="11" width="19.85546875" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="12" max="12" width="15.42578125" style="9" customWidth="1" collapsed="1"/>
-    <col min="13" max="13" width="10.42578125" customWidth="1"/>
-    <col min="14" max="14" width="14.5703125" customWidth="1"/>
-    <col min="15" max="28" width="10.42578125" customWidth="1"/>
-    <col min="29" max="30" width="10.42578125" hidden="1" customWidth="1"/>
-    <col min="31" max="34" width="10.42578125" customWidth="1"/>
-    <col min="35" max="36" width="15.140625" customWidth="1"/>
-    <col min="37" max="37" width="15.85546875" customWidth="1"/>
-    <col min="38" max="39" width="9.5703125" customWidth="1"/>
-    <col min="40" max="41" width="15.42578125" customWidth="1"/>
-    <col min="42" max="42" width="10.42578125" customWidth="1" collapsed="1"/>
-    <col min="43" max="49" width="10.42578125" customWidth="1"/>
-    <col min="50" max="50" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="13.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="13.26953125" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="10" width="12.54296875" style="9" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="19.81640625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="12" max="12" width="15.453125" style="9" customWidth="1" collapsed="1"/>
+    <col min="13" max="13" width="10.453125" customWidth="1"/>
+    <col min="14" max="14" width="14.54296875" customWidth="1"/>
+    <col min="15" max="28" width="10.453125" customWidth="1"/>
+    <col min="29" max="30" width="10.453125" hidden="1" customWidth="1"/>
+    <col min="31" max="34" width="10.453125" customWidth="1"/>
+    <col min="35" max="36" width="15.1796875" customWidth="1"/>
+    <col min="37" max="37" width="15.81640625" customWidth="1"/>
+    <col min="38" max="39" width="9.54296875" customWidth="1"/>
+    <col min="40" max="41" width="15.453125" customWidth="1"/>
+    <col min="42" max="42" width="10.453125" customWidth="1" collapsed="1"/>
+    <col min="43" max="49" width="10.453125" customWidth="1"/>
+    <col min="50" max="50" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="13.26953125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:58" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:58" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>5</v>
       </c>
@@ -1755,7 +1752,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
         <v>60</v>
       </c>
@@ -1928,7 +1925,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="3" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
         <v>120</v>
       </c>
@@ -2101,7 +2098,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="4" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
         <v>121</v>
       </c>
@@ -2274,7 +2271,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="5" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>233</v>
       </c>
@@ -2447,7 +2444,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="6" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>416</v>
       </c>
@@ -2620,7 +2617,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="7" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>752</v>
       </c>
@@ -2791,7 +2788,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="8" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>761</v>
       </c>
@@ -2961,7 +2958,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="9" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>888</v>
       </c>
@@ -3133,7 +3130,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="10" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>901</v>
       </c>
@@ -3306,7 +3303,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="11" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>904</v>
       </c>
@@ -3479,7 +3476,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="12" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>906</v>
       </c>
@@ -3652,7 +3649,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="13" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>907</v>
       </c>
@@ -3825,7 +3822,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="14" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>908</v>
       </c>
@@ -3998,7 +3995,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="15" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>910</v>
       </c>
@@ -4172,7 +4169,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="16" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>912</v>
       </c>
@@ -4345,7 +4342,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="17" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>915</v>
       </c>
@@ -4517,7 +4514,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="18" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>916</v>
       </c>
@@ -4690,7 +4687,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="19" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>917</v>
       </c>
@@ -4863,7 +4860,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="20" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>918</v>
       </c>
@@ -5036,7 +5033,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="21" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>920</v>
       </c>
@@ -5209,7 +5206,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="22" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>921</v>
       </c>
@@ -5382,7 +5379,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="23" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>924</v>
       </c>
@@ -5555,7 +5552,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="24" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>925</v>
       </c>
@@ -5728,7 +5725,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="25" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>927</v>
       </c>
@@ -5901,7 +5898,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="26" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>928</v>
       </c>
@@ -6074,7 +6071,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="27" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>930</v>
       </c>
@@ -6246,7 +6243,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="28" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:51" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>931</v>
       </c>
@@ -6419,7 +6416,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="29" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>932</v>
       </c>
@@ -6592,7 +6589,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="30" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>1005</v>
       </c>
@@ -6764,7 +6761,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="31" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>1006</v>
       </c>
@@ -6936,7 +6933,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="32" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>1007</v>
       </c>
@@ -7110,7 +7107,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="33" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>1009</v>
       </c>
@@ -7282,7 +7279,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="34" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>1010</v>
       </c>
@@ -7454,7 +7451,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="35" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
         <v>1012</v>
       </c>
@@ -7627,7 +7624,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="36" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
         <v>1014</v>
       </c>
@@ -7799,7 +7796,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="37" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
         <v>1015</v>
       </c>
@@ -7971,7 +7968,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="38" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
         <v>1034</v>
       </c>
@@ -8143,7 +8140,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="39" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
         <v>1036</v>
       </c>
@@ -8315,7 +8312,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="40" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
         <v>1037</v>
       </c>
@@ -8487,7 +8484,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="41" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
         <v>1039</v>
       </c>
@@ -8660,7 +8657,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="42" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
         <v>1040</v>
       </c>
@@ -8832,7 +8829,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="43" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
         <v>1045</v>
       </c>
@@ -9005,7 +9002,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="44" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
         <v>1084</v>
       </c>
@@ -9178,7 +9175,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="45" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:51" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
         <v>138</v>
       </c>
@@ -9340,9 +9337,9 @@
         <v>46508</v>
       </c>
     </row>
-    <row r="46" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:51" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>80</v>
@@ -9502,7 +9499,7 @@
         <v>46508</v>
       </c>
     </row>
-    <row r="47" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
         <v>143</v>
       </c>
@@ -9588,7 +9585,7 @@
         <v>31</v>
       </c>
       <c r="Z47" s="6">
-        <f t="shared" ref="Z46:Z52" si="49">+Y47+X47-1</f>
+        <f t="shared" ref="Z47:Z51" si="49">+Y47+X47-1</f>
         <v>33</v>
       </c>
       <c r="AA47" s="6">
@@ -9677,7 +9674,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="48" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>144</v>
       </c>
@@ -9691,7 +9688,7 @@
         <v>77</v>
       </c>
       <c r="E48" s="38" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F48" s="19">
         <v>90012500</v>
@@ -9849,7 +9846,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="49" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
         <v>145</v>
       </c>
@@ -10018,11 +10015,11 @@
       <c r="AX49" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="AY49" s="41">
+      <c r="AY49" s="40">
         <v>46507</v>
       </c>
     </row>
-    <row r="50" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>146</v>
       </c>
@@ -10197,7 +10194,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="51" spans="1:51" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:51" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>147</v>
       </c>
@@ -10372,7 +10369,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="52" spans="1:51" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:51" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>152</v>
       </c>
@@ -10542,11 +10539,11 @@
       <c r="AX52" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="AY52" s="41">
+      <c r="AY52" s="40">
         <v>46507</v>
       </c>
     </row>
-    <row r="53" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:51" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>168</v>
       </c>
@@ -10711,7 +10708,14 @@
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
-  <autoFilter ref="A1:AY53" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}"/>
+  <autoFilter ref="A1:AY53" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="O001"/>
+        <filter val="O010"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="8" type="noConversion"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:E12 K2:K12 K16:K1048195 C16:E1048195" xr:uid="{833F6030-824F-4AAE-BA3C-131D886541AF}">
@@ -10736,9 +10740,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7007F1-B98C-4FB4-AD1E-FC672D1A14BF}">
   <dimension ref="B2:E5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>161</v>
       </c>
@@ -10752,7 +10756,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>164</v>
       </c>
@@ -10766,7 +10770,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>167</v>
       </c>

</xml_diff>

<commit_message>
930 + simulaciones S
</commit_message>
<xml_diff>
--- a/VTT Tool/VTT DATA.xlsx
+++ b/VTT Tool/VTT DATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOJorge\Documents\Python projects\Horse Luis\VTT Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAD0B8B9-3AC4-4CDC-B54E-88F8E53200E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC07925-F144-47AB-AB15-F42C57458940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="190" yWindow="260" windowWidth="19010" windowHeight="11370" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
   </bookViews>
   <sheets>
     <sheet name="VTT actif" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Hoja2!$D$7:$H$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'VTT actif'!$A$1:$AY$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'VTT actif'!$A$1:$AY$57</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -427,7 +427,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="180">
   <si>
     <t>Compte Consignee</t>
   </si>
@@ -952,6 +952,21 @@
   </si>
   <si>
     <t>Customs (days)</t>
+  </si>
+  <si>
+    <t>NITCO</t>
+  </si>
+  <si>
+    <t>O011</t>
+  </si>
+  <si>
+    <t>S001</t>
+  </si>
+  <si>
+    <t>HUIWANG</t>
+  </si>
+  <si>
+    <t>S002</t>
   </si>
 </sst>
 </file>
@@ -1183,7 +1198,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1325,6 +1340,9 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1671,18 +1689,16 @@
     <col min="2" max="2" width="12.85546875" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="10.42578125" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" style="9" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="7" max="7" width="15.42578125" style="8" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="8" max="8" width="16" style="8" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="9" max="9" width="13.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="10" max="10" width="12.5703125" style="9" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="11" width="19.85546875" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="12" max="12" width="15.42578125" style="9" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="12.42578125" style="9" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="15.42578125" style="8" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="16" style="8" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="13.28515625" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="10" width="12.5703125" style="9" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="19.85546875" customWidth="1" outlineLevel="1"/>
+    <col min="12" max="12" width="15.42578125" style="9" customWidth="1"/>
     <col min="13" max="13" width="10.42578125" customWidth="1"/>
     <col min="14" max="14" width="14.5703125" customWidth="1"/>
-    <col min="15" max="28" width="10.42578125" customWidth="1"/>
-    <col min="29" max="30" width="10.42578125" hidden="1" customWidth="1"/>
-    <col min="31" max="34" width="10.42578125" customWidth="1"/>
+    <col min="15" max="34" width="10.42578125" customWidth="1"/>
     <col min="35" max="36" width="15.140625" customWidth="1"/>
     <col min="37" max="37" width="15.85546875" customWidth="1"/>
     <col min="38" max="39" width="9.5703125" customWidth="1"/>
@@ -1909,7 +1925,7 @@
         <v>15</v>
       </c>
       <c r="P2" s="3">
-        <f t="shared" ref="P2:P40" si="0">+IF(I2="SFK Freight Forwarder",0,5)</f>
+        <f t="shared" ref="P2:P26" si="0">+IF(I2="SFK Freight Forwarder",0,5)</f>
         <v>5</v>
       </c>
       <c r="Q2" s="3">
@@ -4622,7 +4638,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="18" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>916</v>
       </c>
@@ -4968,7 +4984,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="20" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>918</v>
       </c>
@@ -5141,39 +5157,39 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="21" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>1039</v>
+        <v>920</v>
       </c>
       <c r="B21" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D21" s="6" t="s">
+      <c r="C21" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="D21" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="33" t="s">
         <v>81</v>
       </c>
       <c r="F21" s="19">
-        <v>91017700</v>
-      </c>
-      <c r="G21" s="5" t="s">
+        <v>91017500</v>
+      </c>
+      <c r="G21" s="35" t="s">
         <v>157</v>
       </c>
       <c r="H21" s="2">
-        <v>222222</v>
+        <v>2533780535</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="J21" s="2">
-        <v>222222</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>46</v>
+        <v>2533780535</v>
+      </c>
+      <c r="K21" s="44" t="s">
+        <v>22</v>
       </c>
       <c r="L21" s="3">
         <v>7</v>
@@ -5183,11 +5199,11 @@
         <v>9</v>
       </c>
       <c r="N21" s="3">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="O21" s="3">
         <f t="shared" si="15"/>
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="P21" s="3">
         <f t="shared" si="0"/>
@@ -5195,111 +5211,111 @@
       </c>
       <c r="Q21" s="3">
         <f t="shared" si="1"/>
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="R21" s="3">
         <f t="shared" si="16"/>
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="S21" s="3">
         <v>7</v>
       </c>
       <c r="T21" s="3">
         <f t="shared" si="2"/>
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="U21" s="3">
         <f t="shared" si="3"/>
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="V21" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W21" s="3">
         <f t="shared" si="4"/>
+        <v>32</v>
+      </c>
+      <c r="X21" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="3">
+        <v>33</v>
+      </c>
+      <c r="Z21" s="6">
         <v>37</v>
-      </c>
-      <c r="X21" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y21" s="3">
-        <v>37</v>
-      </c>
-      <c r="Z21" s="6">
-        <v>42</v>
       </c>
       <c r="AA21" s="6">
         <f t="shared" si="19"/>
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="AB21" s="3">
         <v>3</v>
       </c>
       <c r="AC21" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AD21" s="3">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="AE21" s="3">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="AF21" s="3">
         <f t="shared" si="6"/>
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AG21" s="6">
         <v>3</v>
       </c>
       <c r="AH21" s="6">
         <f t="shared" si="7"/>
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="AI21" s="3">
         <v>0</v>
       </c>
       <c r="AJ21" s="3">
         <f t="shared" si="8"/>
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="AK21" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="AL21" s="3">
+      <c r="AL21" s="46">
         <v>2</v>
       </c>
       <c r="AM21" s="3">
         <f t="shared" si="9"/>
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="AN21" s="3">
         <v>8</v>
       </c>
       <c r="AO21" s="3">
         <f t="shared" si="10"/>
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="AP21" s="3">
         <v>2</v>
       </c>
       <c r="AQ21" s="3">
         <f t="shared" si="11"/>
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="AR21" s="3">
         <f t="shared" si="12"/>
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="AS21" s="3">
         <f t="shared" si="13"/>
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="AT21" s="3">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="AU21" s="3">
         <f t="shared" si="14"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AV21" s="3" t="s">
         <v>130</v>
@@ -5308,7 +5324,7 @@
         <v>131</v>
       </c>
       <c r="AX21" s="20" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="AY21" s="21">
         <v>46507</v>
@@ -6181,13 +6197,13 @@
     </row>
     <row r="27" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
-        <v>920</v>
+        <v>930</v>
       </c>
       <c r="B27" s="33" t="s">
         <v>80</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D27" s="33" t="s">
         <v>58</v>
@@ -6196,22 +6212,22 @@
         <v>81</v>
       </c>
       <c r="F27" s="19">
-        <v>91017500</v>
-      </c>
-      <c r="G27" s="35" t="s">
+        <v>91017700</v>
+      </c>
+      <c r="G27" s="4" t="s">
         <v>157</v>
       </c>
       <c r="H27" s="2">
-        <v>2533780535</v>
+        <v>26037000</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="J27" s="2">
-        <v>2533780535</v>
-      </c>
-      <c r="K27" s="44" t="s">
-        <v>22</v>
+        <v>26037000</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="L27" s="3">
         <v>7</v>
@@ -6228,7 +6244,6 @@
         <v>22</v>
       </c>
       <c r="P27" s="3">
-        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="Q27" s="3">
@@ -6251,54 +6266,54 @@
         <v>30</v>
       </c>
       <c r="V27" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W27" s="3">
         <f t="shared" si="4"/>
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="X27" s="3">
         <v>0</v>
       </c>
       <c r="Y27" s="3">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="Z27" s="6">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="AA27" s="6">
         <f t="shared" si="19"/>
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AB27" s="3">
         <v>3</v>
       </c>
       <c r="AC27" s="3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AD27" s="3">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="AE27" s="3">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="AF27" s="3">
         <f t="shared" si="6"/>
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AG27" s="6">
         <v>3</v>
       </c>
       <c r="AH27" s="6">
         <f t="shared" si="7"/>
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AI27" s="3">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AJ27" s="3">
         <f t="shared" si="8"/>
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="AK27" s="3" t="s">
         <v>55</v>
@@ -6308,36 +6323,36 @@
       </c>
       <c r="AM27" s="3">
         <f t="shared" si="9"/>
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="AN27" s="3">
         <v>8</v>
       </c>
       <c r="AO27" s="3">
         <f t="shared" si="10"/>
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="AP27" s="3">
         <v>2</v>
       </c>
       <c r="AQ27" s="3">
         <f t="shared" si="11"/>
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="AR27" s="3">
         <f t="shared" si="12"/>
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="AS27" s="3">
         <f t="shared" si="13"/>
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="AT27" s="3">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="AU27" s="3">
         <f t="shared" si="14"/>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AV27" s="3" t="s">
         <v>130</v>
@@ -6401,7 +6416,7 @@
         <v>22</v>
       </c>
       <c r="P28" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="P28:P44" si="20">+IF(I28="SFK Freight Forwarder",0,5)</f>
         <v>5</v>
       </c>
       <c r="Q28" s="3">
@@ -6574,7 +6589,7 @@
         <v>22</v>
       </c>
       <c r="P29" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>5</v>
       </c>
       <c r="Q29" s="3">
@@ -6746,7 +6761,7 @@
         <v>0</v>
       </c>
       <c r="P30" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q30" s="3">
@@ -6918,7 +6933,7 @@
         <v>0</v>
       </c>
       <c r="P31" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q31" s="3">
@@ -7090,7 +7105,7 @@
         <v>0</v>
       </c>
       <c r="P32" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q32" s="3">
@@ -7264,7 +7279,7 @@
         <v>0</v>
       </c>
       <c r="P33" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q33" s="3">
@@ -7436,11 +7451,11 @@
         <v>0</v>
       </c>
       <c r="P34" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q34" s="3">
-        <f t="shared" ref="Q34:Q65" si="20">+IF(I34="SFK Freight Forwarder",O34,O34+P34-1)</f>
+        <f t="shared" ref="Q34:Q65" si="21">+IF(I34="SFK Freight Forwarder",O34,O34+P34-1)</f>
         <v>0</v>
       </c>
       <c r="R34" s="3">
@@ -7451,7 +7466,7 @@
         <v>7</v>
       </c>
       <c r="T34" s="3">
-        <f t="shared" ref="T34:T65" si="21">+R34+S34-1</f>
+        <f t="shared" ref="T34:T65" si="22">+R34+S34-1</f>
         <v>29</v>
       </c>
       <c r="U34" s="3">
@@ -7462,7 +7477,7 @@
         <v>1</v>
       </c>
       <c r="W34" s="3">
-        <f t="shared" ref="W34:W65" si="22">+U34+V34-1</f>
+        <f t="shared" ref="W34:W65" si="23">+U34+V34-1</f>
         <v>30</v>
       </c>
       <c r="X34" s="3">
@@ -7491,21 +7506,21 @@
         <v>63</v>
       </c>
       <c r="AF34" s="3">
-        <f t="shared" ref="AF34:AF65" si="23">+AE34+AA34-1</f>
+        <f t="shared" ref="AF34:AF65" si="24">+AE34+AA34-1</f>
         <v>98</v>
       </c>
       <c r="AG34" s="6">
         <v>3</v>
       </c>
       <c r="AH34" s="6">
-        <f t="shared" ref="AH34:AH65" si="24">+AF34+AG34</f>
+        <f t="shared" ref="AH34:AH65" si="25">+AF34+AG34</f>
         <v>101</v>
       </c>
       <c r="AI34" s="3">
         <v>0</v>
       </c>
       <c r="AJ34" s="3">
-        <f t="shared" ref="AJ34:AJ65" si="25">+AI34+AH34</f>
+        <f t="shared" ref="AJ34:AJ65" si="26">+AI34+AH34</f>
         <v>101</v>
       </c>
       <c r="AK34" s="3" t="s">
@@ -7515,14 +7530,14 @@
         <v>4</v>
       </c>
       <c r="AM34" s="3">
-        <f t="shared" ref="AM34:AM65" si="26">+AJ34+AL34</f>
+        <f t="shared" ref="AM34:AM65" si="27">+AJ34+AL34</f>
         <v>105</v>
       </c>
       <c r="AN34" s="3">
         <v>3</v>
       </c>
       <c r="AO34" s="3">
-        <f t="shared" ref="AO34:AO65" si="27">+AM34+AN34</f>
+        <f t="shared" ref="AO34:AO65" si="28">+AM34+AN34</f>
         <v>108</v>
       </c>
       <c r="AP34" s="3">
@@ -7537,14 +7552,14 @@
         <v>119</v>
       </c>
       <c r="AS34" s="3">
-        <f t="shared" ref="AS34:AS65" si="28">+AR34+7+AT34</f>
+        <f t="shared" ref="AS34:AS65" si="29">+AR34+7+AT34</f>
         <v>126</v>
       </c>
       <c r="AT34" s="3">
         <v>0</v>
       </c>
       <c r="AU34" s="3">
-        <f t="shared" ref="AU34:AU54" si="29">+AA34-R34</f>
+        <f t="shared" ref="AU34:AU55" si="30">+AA34-R34</f>
         <v>13</v>
       </c>
       <c r="AV34" s="3" t="s">
@@ -7608,11 +7623,11 @@
         <v>0</v>
       </c>
       <c r="P35" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q35" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="R35" s="3">
@@ -7623,7 +7638,7 @@
         <v>7</v>
       </c>
       <c r="T35" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U35" s="3">
@@ -7634,7 +7649,7 @@
         <v>1</v>
       </c>
       <c r="W35" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>30</v>
       </c>
       <c r="X35" s="3">
@@ -7664,21 +7679,21 @@
         <v>48</v>
       </c>
       <c r="AF35" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>84</v>
       </c>
       <c r="AG35" s="6">
         <v>3</v>
       </c>
       <c r="AH35" s="6">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>87</v>
       </c>
       <c r="AI35" s="3">
         <v>14</v>
       </c>
       <c r="AJ35" s="3">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>101</v>
       </c>
       <c r="AK35" s="3" t="s">
@@ -7688,14 +7703,14 @@
         <v>2</v>
       </c>
       <c r="AM35" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>103</v>
       </c>
       <c r="AN35" s="3">
         <v>2</v>
       </c>
       <c r="AO35" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>105</v>
       </c>
       <c r="AP35" s="3">
@@ -7710,14 +7725,14 @@
         <v>112</v>
       </c>
       <c r="AS35" s="3">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>119</v>
       </c>
       <c r="AT35" s="3">
         <v>0</v>
       </c>
       <c r="AU35" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>14</v>
       </c>
       <c r="AV35" s="3" t="s">
@@ -7781,11 +7796,11 @@
         <v>0</v>
       </c>
       <c r="P36" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q36" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="R36" s="3">
@@ -7796,7 +7811,7 @@
         <v>7</v>
       </c>
       <c r="T36" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U36" s="3">
@@ -7807,7 +7822,7 @@
         <v>2</v>
       </c>
       <c r="W36" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>31</v>
       </c>
       <c r="X36" s="3">
@@ -7836,23 +7851,23 @@
         <v>17</v>
       </c>
       <c r="AF36" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>60</v>
       </c>
       <c r="AG36" s="6">
         <v>3</v>
       </c>
       <c r="AH36" s="6">
-        <f t="shared" si="24"/>
-        <v>63</v>
-      </c>
-      <c r="AI36" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ36" s="3">
         <f t="shared" si="25"/>
         <v>63</v>
       </c>
+      <c r="AI36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ36" s="3">
+        <f t="shared" si="26"/>
+        <v>63</v>
+      </c>
       <c r="AK36" s="3" t="s">
         <v>60</v>
       </c>
@@ -7860,14 +7875,14 @@
         <v>0</v>
       </c>
       <c r="AM36" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>63</v>
       </c>
       <c r="AN36" s="3">
         <v>0</v>
       </c>
       <c r="AO36" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>63</v>
       </c>
       <c r="AP36" s="3">
@@ -7882,14 +7897,14 @@
         <v>70</v>
       </c>
       <c r="AS36" s="3">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>77</v>
       </c>
       <c r="AT36" s="3">
         <v>0</v>
       </c>
       <c r="AU36" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>21</v>
       </c>
       <c r="AV36" s="3" t="s">
@@ -7953,11 +7968,11 @@
         <v>0</v>
       </c>
       <c r="P37" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q37" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="R37" s="3">
@@ -7968,7 +7983,7 @@
         <v>7</v>
       </c>
       <c r="T37" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U37" s="3">
@@ -7979,7 +7994,7 @@
         <v>2</v>
       </c>
       <c r="W37" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>31</v>
       </c>
       <c r="X37" s="3">
@@ -8008,23 +8023,23 @@
         <v>34</v>
       </c>
       <c r="AF37" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>77</v>
       </c>
       <c r="AG37" s="6">
         <v>3</v>
       </c>
       <c r="AH37" s="6">
-        <f t="shared" si="24"/>
-        <v>80</v>
-      </c>
-      <c r="AI37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ37" s="3">
         <f t="shared" si="25"/>
         <v>80</v>
       </c>
+      <c r="AI37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ37" s="3">
+        <f t="shared" si="26"/>
+        <v>80</v>
+      </c>
       <c r="AK37" s="3" t="s">
         <v>60</v>
       </c>
@@ -8032,14 +8047,14 @@
         <v>2</v>
       </c>
       <c r="AM37" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>82</v>
       </c>
       <c r="AN37" s="3">
         <v>2</v>
       </c>
       <c r="AO37" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>84</v>
       </c>
       <c r="AP37" s="3">
@@ -8054,14 +8069,14 @@
         <v>91</v>
       </c>
       <c r="AS37" s="3">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>98</v>
       </c>
       <c r="AT37" s="3">
         <v>0</v>
       </c>
       <c r="AU37" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>21</v>
       </c>
       <c r="AV37" s="3" t="s">
@@ -8125,11 +8140,11 @@
         <v>0</v>
       </c>
       <c r="P38" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q38" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="R38" s="3">
@@ -8140,7 +8155,7 @@
         <v>7</v>
       </c>
       <c r="T38" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U38" s="3">
@@ -8151,7 +8166,7 @@
         <v>1</v>
       </c>
       <c r="W38" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>30</v>
       </c>
       <c r="X38" s="3">
@@ -8180,23 +8195,23 @@
         <v>53</v>
       </c>
       <c r="AF38" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>87</v>
       </c>
       <c r="AG38" s="6">
         <v>3</v>
       </c>
       <c r="AH38" s="6">
-        <f t="shared" si="24"/>
-        <v>90</v>
-      </c>
-      <c r="AI38" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ38" s="3">
         <f t="shared" si="25"/>
         <v>90</v>
       </c>
+      <c r="AI38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ38" s="3">
+        <f t="shared" si="26"/>
+        <v>90</v>
+      </c>
       <c r="AK38" s="3" t="s">
         <v>60</v>
       </c>
@@ -8204,14 +8219,14 @@
         <v>2</v>
       </c>
       <c r="AM38" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>92</v>
       </c>
       <c r="AN38" s="3">
         <v>6</v>
       </c>
       <c r="AO38" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>98</v>
       </c>
       <c r="AP38" s="3">
@@ -8226,14 +8241,14 @@
         <v>105</v>
       </c>
       <c r="AS38" s="3">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>112</v>
       </c>
       <c r="AT38" s="3">
         <v>0</v>
       </c>
       <c r="AU38" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>12</v>
       </c>
       <c r="AV38" s="3" t="s">
@@ -8297,11 +8312,11 @@
         <v>0</v>
       </c>
       <c r="P39" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q39" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="R39" s="3">
@@ -8312,7 +8327,7 @@
         <v>7</v>
       </c>
       <c r="T39" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U39" s="3">
@@ -8323,7 +8338,7 @@
         <v>2</v>
       </c>
       <c r="W39" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>31</v>
       </c>
       <c r="X39" s="3">
@@ -8352,23 +8367,23 @@
         <v>31</v>
       </c>
       <c r="AF39" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>66</v>
       </c>
       <c r="AG39" s="6">
         <v>3</v>
       </c>
       <c r="AH39" s="6">
-        <f t="shared" si="24"/>
-        <v>69</v>
-      </c>
-      <c r="AI39" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ39" s="3">
         <f t="shared" si="25"/>
         <v>69</v>
       </c>
+      <c r="AI39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ39" s="3">
+        <f t="shared" si="26"/>
+        <v>69</v>
+      </c>
       <c r="AK39" s="3" t="s">
         <v>60</v>
       </c>
@@ -8376,14 +8391,14 @@
         <v>2</v>
       </c>
       <c r="AM39" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>71</v>
       </c>
       <c r="AN39" s="3">
         <v>5</v>
       </c>
       <c r="AO39" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>76</v>
       </c>
       <c r="AP39" s="3">
@@ -8398,14 +8413,14 @@
         <v>84</v>
       </c>
       <c r="AS39" s="3">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>91</v>
       </c>
       <c r="AT39" s="3">
         <v>0</v>
       </c>
       <c r="AU39" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>13</v>
       </c>
       <c r="AV39" s="3" t="s">
@@ -8469,11 +8484,11 @@
         <v>0</v>
       </c>
       <c r="P40" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q40" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="R40" s="3">
@@ -8484,7 +8499,7 @@
         <v>7</v>
       </c>
       <c r="T40" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U40" s="3">
@@ -8495,7 +8510,7 @@
         <v>1</v>
       </c>
       <c r="W40" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>30</v>
       </c>
       <c r="X40" s="3">
@@ -8524,21 +8539,21 @@
         <v>67</v>
       </c>
       <c r="AF40" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>102</v>
       </c>
       <c r="AG40" s="6">
         <v>3</v>
       </c>
       <c r="AH40" s="6">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>105</v>
       </c>
       <c r="AI40" s="3">
         <v>7</v>
       </c>
       <c r="AJ40" s="3">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>112</v>
       </c>
       <c r="AK40" s="3" t="s">
@@ -8548,14 +8563,14 @@
         <v>3</v>
       </c>
       <c r="AM40" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>115</v>
       </c>
       <c r="AN40" s="3">
         <v>3</v>
       </c>
       <c r="AO40" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>118</v>
       </c>
       <c r="AP40" s="3">
@@ -8570,14 +8585,14 @@
         <v>126</v>
       </c>
       <c r="AS40" s="3">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>133</v>
       </c>
       <c r="AT40" s="3">
         <v>0</v>
       </c>
       <c r="AU40" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>13</v>
       </c>
       <c r="AV40" s="3" t="s">
@@ -8593,141 +8608,142 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="41" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>930</v>
+        <v>1039</v>
       </c>
       <c r="B41" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="33" t="s">
+      <c r="C41" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D41" s="33" t="s">
+      <c r="D41" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E41" s="33" t="s">
+      <c r="E41" s="6" t="s">
         <v>81</v>
       </c>
       <c r="F41" s="19">
         <v>91017700</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="G41" s="5" t="s">
         <v>157</v>
       </c>
       <c r="H41" s="2">
-        <v>26037000</v>
+        <v>222222</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="J41" s="2">
-        <v>26037000</v>
+        <v>222222</v>
       </c>
       <c r="K41" s="4" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="L41" s="3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="M41" s="3">
         <f>+IF(I41="SFK Freight Forwarder",L41,9)</f>
         <v>9</v>
       </c>
       <c r="N41" s="3">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="O41" s="3">
         <f t="shared" si="15"/>
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="P41" s="3">
+        <f t="shared" si="20"/>
         <v>5</v>
       </c>
       <c r="Q41" s="3">
-        <f t="shared" si="20"/>
-        <v>26</v>
+        <f t="shared" si="21"/>
+        <v>33</v>
       </c>
       <c r="R41" s="3">
         <f t="shared" si="16"/>
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="S41" s="3">
         <v>7</v>
       </c>
       <c r="T41" s="3">
-        <f t="shared" si="21"/>
-        <v>29</v>
+        <f t="shared" si="22"/>
+        <v>36</v>
       </c>
       <c r="U41" s="3">
         <f t="shared" si="3"/>
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="V41" s="3">
         <v>1</v>
       </c>
       <c r="W41" s="3">
-        <f t="shared" si="22"/>
-        <v>30</v>
+        <f t="shared" si="23"/>
+        <v>37</v>
       </c>
       <c r="X41" s="3">
         <v>0</v>
       </c>
       <c r="Y41" s="3">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="Z41" s="6">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AA41" s="6">
         <f t="shared" si="19"/>
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="AB41" s="3">
         <v>3</v>
       </c>
       <c r="AC41" s="3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AD41" s="3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AE41" s="3">
         <v>40</v>
       </c>
       <c r="AF41" s="3">
-        <f t="shared" si="23"/>
-        <v>76</v>
+        <f t="shared" si="24"/>
+        <v>83</v>
       </c>
       <c r="AG41" s="6">
         <v>3</v>
       </c>
       <c r="AH41" s="6">
-        <f t="shared" si="24"/>
-        <v>79</v>
-      </c>
-      <c r="AI41" s="3">
-        <v>7</v>
-      </c>
-      <c r="AJ41" s="3">
         <f t="shared" si="25"/>
         <v>86</v>
       </c>
+      <c r="AI41" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ41" s="3">
+        <f t="shared" si="26"/>
+        <v>86</v>
+      </c>
       <c r="AK41" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="AL41" s="46">
+      <c r="AL41" s="3">
         <v>2</v>
       </c>
       <c r="AM41" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>88</v>
       </c>
       <c r="AN41" s="3">
         <v>8</v>
       </c>
       <c r="AO41" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>96</v>
       </c>
       <c r="AP41" s="3">
@@ -8742,14 +8758,14 @@
         <v>105</v>
       </c>
       <c r="AS41" s="3">
-        <f t="shared" si="28"/>
-        <v>129</v>
+        <f t="shared" si="29"/>
+        <v>112</v>
       </c>
       <c r="AT41" s="3">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="AU41" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>14</v>
       </c>
       <c r="AV41" s="3" t="s">
@@ -8759,7 +8775,7 @@
         <v>131</v>
       </c>
       <c r="AX41" s="20" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="AY41" s="21">
         <v>46507</v>
@@ -8813,11 +8829,11 @@
         <v>0</v>
       </c>
       <c r="P42" s="3">
-        <f>+IF(I42="SFK Freight Forwarder",0,5)</f>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="Q42" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="R42" s="3">
@@ -8828,7 +8844,7 @@
         <v>7</v>
       </c>
       <c r="T42" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U42" s="3">
@@ -8839,7 +8855,7 @@
         <v>1</v>
       </c>
       <c r="W42" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>30</v>
       </c>
       <c r="X42" s="3">
@@ -8868,23 +8884,23 @@
         <v>32</v>
       </c>
       <c r="AF42" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>67</v>
       </c>
       <c r="AG42" s="6">
         <v>3</v>
       </c>
       <c r="AH42" s="6">
-        <f t="shared" si="24"/>
-        <v>70</v>
-      </c>
-      <c r="AI42" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ42" s="3">
         <f t="shared" si="25"/>
         <v>70</v>
       </c>
+      <c r="AI42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ42" s="3">
+        <f t="shared" si="26"/>
+        <v>70</v>
+      </c>
       <c r="AK42" s="3" t="s">
         <v>60</v>
       </c>
@@ -8892,14 +8908,14 @@
         <v>4</v>
       </c>
       <c r="AM42" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>74</v>
       </c>
       <c r="AN42" s="3">
         <v>3</v>
       </c>
       <c r="AO42" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>77</v>
       </c>
       <c r="AP42" s="3">
@@ -8914,14 +8930,14 @@
         <v>84</v>
       </c>
       <c r="AS42" s="3">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>91</v>
       </c>
       <c r="AT42" s="3">
         <v>0</v>
       </c>
       <c r="AU42" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>13</v>
       </c>
       <c r="AV42" s="3" t="s">
@@ -8986,11 +9002,11 @@
         <v>29</v>
       </c>
       <c r="P43" s="3">
-        <f>+IF(I43="SFK Freight Forwarder",0,5)</f>
+        <f t="shared" si="20"/>
         <v>5</v>
       </c>
       <c r="Q43" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>33</v>
       </c>
       <c r="R43" s="3">
@@ -9001,7 +9017,7 @@
         <v>7</v>
       </c>
       <c r="T43" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>36</v>
       </c>
       <c r="U43" s="3">
@@ -9012,7 +9028,7 @@
         <v>1</v>
       </c>
       <c r="W43" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>37</v>
       </c>
       <c r="X43" s="3">
@@ -9041,21 +9057,21 @@
         <v>46</v>
       </c>
       <c r="AF43" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>84</v>
       </c>
       <c r="AG43" s="6">
         <v>3</v>
       </c>
       <c r="AH43" s="6">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>87</v>
       </c>
       <c r="AI43" s="3">
         <v>7</v>
       </c>
       <c r="AJ43" s="3">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>94</v>
       </c>
       <c r="AK43" s="3" t="s">
@@ -9065,14 +9081,14 @@
         <v>4</v>
       </c>
       <c r="AM43" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>98</v>
       </c>
       <c r="AN43" s="3">
         <v>3</v>
       </c>
       <c r="AO43" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>101</v>
       </c>
       <c r="AP43" s="3">
@@ -9087,14 +9103,14 @@
         <v>112</v>
       </c>
       <c r="AS43" s="3">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>119</v>
       </c>
       <c r="AT43" s="3">
         <v>0</v>
       </c>
       <c r="AU43" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>9</v>
       </c>
       <c r="AV43" s="3" t="s">
@@ -9159,11 +9175,11 @@
         <v>22</v>
       </c>
       <c r="P44" s="3">
-        <f>+IF(I44="SFK Freight Forwarder",0,5)</f>
+        <f t="shared" si="20"/>
         <v>5</v>
       </c>
       <c r="Q44" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>26</v>
       </c>
       <c r="R44" s="3">
@@ -9174,7 +9190,7 @@
         <v>7</v>
       </c>
       <c r="T44" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U44" s="3">
@@ -9185,7 +9201,7 @@
         <v>2</v>
       </c>
       <c r="W44" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>31</v>
       </c>
       <c r="X44" s="3">
@@ -9214,23 +9230,23 @@
         <v>35</v>
       </c>
       <c r="AF44" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>75</v>
       </c>
       <c r="AG44" s="6">
         <v>3</v>
       </c>
       <c r="AH44" s="6">
-        <f t="shared" si="24"/>
-        <v>78</v>
-      </c>
-      <c r="AI44" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ44" s="3">
         <f t="shared" si="25"/>
         <v>78</v>
       </c>
+      <c r="AI44" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ44" s="3">
+        <f t="shared" si="26"/>
+        <v>78</v>
+      </c>
       <c r="AK44" s="3" t="s">
         <v>65</v>
       </c>
@@ -9238,14 +9254,14 @@
         <v>2</v>
       </c>
       <c r="AM44" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>80</v>
       </c>
       <c r="AN44" s="3">
         <v>2</v>
       </c>
       <c r="AO44" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>82</v>
       </c>
       <c r="AP44" s="3">
@@ -9260,14 +9276,14 @@
         <v>91</v>
       </c>
       <c r="AS44" s="3">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>98</v>
       </c>
       <c r="AT44" s="3">
         <v>0</v>
       </c>
       <c r="AU44" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>18</v>
       </c>
       <c r="AV44" s="3" t="s">
@@ -9334,7 +9350,7 @@
         <v>6</v>
       </c>
       <c r="Q45" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>13</v>
       </c>
       <c r="R45" s="23">
@@ -9344,7 +9360,7 @@
         <v>12</v>
       </c>
       <c r="T45" s="23">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>20</v>
       </c>
       <c r="U45" s="23">
@@ -9355,7 +9371,7 @@
         <v>5</v>
       </c>
       <c r="W45" s="23">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>26</v>
       </c>
       <c r="X45" s="23">
@@ -9379,21 +9395,21 @@
         <v>41</v>
       </c>
       <c r="AF45" s="23">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>71</v>
       </c>
       <c r="AG45" s="23">
         <v>3</v>
       </c>
       <c r="AH45" s="23">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>74</v>
       </c>
       <c r="AI45" s="23">
         <v>7</v>
       </c>
       <c r="AJ45" s="23">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>81</v>
       </c>
       <c r="AK45" s="23"/>
@@ -9401,14 +9417,14 @@
         <v>3</v>
       </c>
       <c r="AM45" s="23">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>84</v>
       </c>
       <c r="AN45" s="23">
         <v>5</v>
       </c>
       <c r="AO45" s="23">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>89</v>
       </c>
       <c r="AP45" s="23">
@@ -9422,14 +9438,14 @@
         <v>96</v>
       </c>
       <c r="AS45" s="23">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>117</v>
       </c>
       <c r="AT45" s="23">
         <v>14</v>
       </c>
       <c r="AU45" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>22</v>
       </c>
       <c r="AV45" s="23" t="s">
@@ -9445,7 +9461,7 @@
         <v>46508</v>
       </c>
     </row>
-    <row r="46" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>172</v>
       </c>
@@ -9496,7 +9512,7 @@
         <v>6</v>
       </c>
       <c r="Q46" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>13</v>
       </c>
       <c r="R46" s="23">
@@ -9506,7 +9522,7 @@
         <v>12</v>
       </c>
       <c r="T46" s="23">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>20</v>
       </c>
       <c r="U46" s="23">
@@ -9517,7 +9533,7 @@
         <v>5</v>
       </c>
       <c r="W46" s="23">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>26</v>
       </c>
       <c r="X46" s="23">
@@ -9541,21 +9557,21 @@
         <v>34</v>
       </c>
       <c r="AF46" s="23">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>69</v>
       </c>
       <c r="AG46" s="23">
         <v>3</v>
       </c>
       <c r="AH46" s="23">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>72</v>
       </c>
       <c r="AI46" s="23">
         <v>0</v>
       </c>
       <c r="AJ46" s="23">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>72</v>
       </c>
       <c r="AK46" s="23"/>
@@ -9563,21 +9579,21 @@
         <v>2</v>
       </c>
       <c r="AM46" s="23">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>74</v>
       </c>
       <c r="AN46" s="23">
         <v>1</v>
       </c>
       <c r="AO46" s="23">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>75</v>
       </c>
       <c r="AP46" s="23">
         <v>3</v>
       </c>
       <c r="AQ46" s="3">
-        <f t="shared" ref="AQ46:AQ54" si="30">+AO46+AP46</f>
+        <f t="shared" ref="AQ46:AQ57" si="31">+AO46+AP46</f>
         <v>78</v>
       </c>
       <c r="AR46" s="23">
@@ -9585,14 +9601,14 @@
         <v>82</v>
       </c>
       <c r="AS46" s="23">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>103</v>
       </c>
       <c r="AT46" s="23">
         <v>14</v>
       </c>
       <c r="AU46" s="3">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>27</v>
       </c>
       <c r="AV46" s="23" t="s">
@@ -9646,7 +9662,7 @@
         <v>7</v>
       </c>
       <c r="M47" s="3">
-        <f t="shared" ref="M47:M54" si="31">+IF(I47="SFK Freight Forwarder",L47,9)</f>
+        <f t="shared" ref="M47:M54" si="32">+IF(I47="SFK Freight Forwarder",L47,9)</f>
         <v>9</v>
       </c>
       <c r="N47" s="3">
@@ -9657,33 +9673,33 @@
         <v>22</v>
       </c>
       <c r="P47" s="3">
-        <f t="shared" ref="P47:P52" si="32">+IF(I47="SFK Freight Forwarder",0,5)</f>
+        <f t="shared" ref="P47:P52" si="33">+IF(I47="SFK Freight Forwarder",0,5)</f>
         <v>5</v>
       </c>
       <c r="Q47" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>26</v>
       </c>
       <c r="R47" s="3">
-        <f t="shared" ref="R47:R52" si="33">9+N47</f>
+        <f t="shared" ref="R47:R52" si="34">9+N47</f>
         <v>23</v>
       </c>
       <c r="S47" s="3">
         <v>7</v>
       </c>
       <c r="T47" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U47" s="3">
-        <f t="shared" ref="U47:U52" si="34">+T47+1</f>
+        <f t="shared" ref="U47:U52" si="35">+T47+1</f>
         <v>30</v>
       </c>
       <c r="V47" s="3">
         <v>2</v>
       </c>
       <c r="W47" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>31</v>
       </c>
       <c r="X47" s="3">
@@ -9714,23 +9730,23 @@
         <v>40</v>
       </c>
       <c r="AF47" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>73</v>
       </c>
       <c r="AG47" s="6">
         <v>3</v>
       </c>
       <c r="AH47" s="6">
-        <f t="shared" si="24"/>
-        <v>76</v>
-      </c>
-      <c r="AI47" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ47" s="3">
         <f t="shared" si="25"/>
         <v>76</v>
       </c>
+      <c r="AI47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ47" s="3">
+        <f t="shared" si="26"/>
+        <v>76</v>
+      </c>
       <c r="AK47" s="3" t="s">
         <v>60</v>
       </c>
@@ -9738,36 +9754,36 @@
         <v>2</v>
       </c>
       <c r="AM47" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>78</v>
       </c>
       <c r="AN47" s="3">
         <v>2</v>
       </c>
       <c r="AO47" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>80</v>
       </c>
       <c r="AP47" s="3">
         <v>6</v>
       </c>
       <c r="AQ47" s="3">
+        <f t="shared" si="31"/>
+        <v>86</v>
+      </c>
+      <c r="AR47" s="3">
+        <f t="shared" ref="AR47:AR57" si="36">+AQ47+7</f>
+        <v>93</v>
+      </c>
+      <c r="AS47" s="3">
+        <f t="shared" si="29"/>
+        <v>100</v>
+      </c>
+      <c r="AT47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU47" s="3">
         <f t="shared" si="30"/>
-        <v>86</v>
-      </c>
-      <c r="AR47" s="3">
-        <f t="shared" ref="AR47:AR54" si="35">+AQ47+7</f>
-        <v>93</v>
-      </c>
-      <c r="AS47" s="3">
-        <f t="shared" si="28"/>
-        <v>100</v>
-      </c>
-      <c r="AT47" s="3">
-        <v>0</v>
-      </c>
-      <c r="AU47" s="3">
-        <f t="shared" si="29"/>
         <v>11</v>
       </c>
       <c r="AV47" s="3" t="s">
@@ -9821,7 +9837,7 @@
         <v>7</v>
       </c>
       <c r="M48" s="3">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>9</v>
       </c>
       <c r="N48" s="3">
@@ -9832,33 +9848,33 @@
         <v>22</v>
       </c>
       <c r="P48" s="3">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>5</v>
       </c>
       <c r="Q48" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>26</v>
       </c>
       <c r="R48" s="3">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>23</v>
       </c>
       <c r="S48" s="3">
         <v>7</v>
       </c>
       <c r="T48" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U48" s="3">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>30</v>
       </c>
       <c r="V48" s="3">
         <v>2</v>
       </c>
       <c r="W48" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>31</v>
       </c>
       <c r="X48" s="3">
@@ -9886,23 +9902,23 @@
         <v>68</v>
       </c>
       <c r="AF48" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>103</v>
       </c>
       <c r="AG48" s="6">
         <v>3</v>
       </c>
       <c r="AH48" s="6">
-        <f t="shared" si="24"/>
-        <v>106</v>
-      </c>
-      <c r="AI48" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ48" s="3">
         <f t="shared" si="25"/>
         <v>106</v>
       </c>
+      <c r="AI48" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ48" s="3">
+        <f t="shared" si="26"/>
+        <v>106</v>
+      </c>
       <c r="AK48" s="3" t="s">
         <v>60</v>
       </c>
@@ -9910,36 +9926,36 @@
         <v>2</v>
       </c>
       <c r="AM48" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>108</v>
       </c>
       <c r="AN48" s="3">
         <v>7</v>
       </c>
       <c r="AO48" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>115</v>
       </c>
       <c r="AP48" s="3">
         <v>5</v>
       </c>
       <c r="AQ48" s="3">
+        <f t="shared" si="31"/>
+        <v>120</v>
+      </c>
+      <c r="AR48" s="3">
+        <f t="shared" si="36"/>
+        <v>127</v>
+      </c>
+      <c r="AS48" s="3">
+        <f t="shared" si="29"/>
+        <v>134</v>
+      </c>
+      <c r="AT48" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU48" s="3">
         <f t="shared" si="30"/>
-        <v>120</v>
-      </c>
-      <c r="AR48" s="3">
-        <f t="shared" si="35"/>
-        <v>127</v>
-      </c>
-      <c r="AS48" s="3">
-        <f t="shared" si="28"/>
-        <v>134</v>
-      </c>
-      <c r="AT48" s="3">
-        <v>0</v>
-      </c>
-      <c r="AU48" s="3">
-        <f t="shared" si="29"/>
         <v>13</v>
       </c>
       <c r="AV48" s="3" t="s">
@@ -9955,7 +9971,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="49" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>145</v>
       </c>
@@ -9993,7 +10009,7 @@
         <v>7</v>
       </c>
       <c r="M49" s="3">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>9</v>
       </c>
       <c r="N49" s="3">
@@ -10004,33 +10020,33 @@
         <v>22</v>
       </c>
       <c r="P49" s="3">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>5</v>
       </c>
       <c r="Q49" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>26</v>
       </c>
       <c r="R49" s="3">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>23</v>
       </c>
       <c r="S49" s="3">
         <v>7</v>
       </c>
       <c r="T49" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U49" s="3">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>30</v>
       </c>
       <c r="V49" s="3">
         <v>2</v>
       </c>
       <c r="W49" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>31</v>
       </c>
       <c r="X49" s="3">
@@ -10043,7 +10059,7 @@
         <v>33</v>
       </c>
       <c r="AA49" s="6">
-        <f t="shared" ref="AA49:AA54" si="36">+Z49+AB49-1</f>
+        <f t="shared" ref="AA49:AA54" si="37">+Z49+AB49-1</f>
         <v>38</v>
       </c>
       <c r="AB49" s="3">
@@ -10059,23 +10075,23 @@
         <v>42</v>
       </c>
       <c r="AF49" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>79</v>
       </c>
       <c r="AG49" s="6">
         <v>3</v>
       </c>
       <c r="AH49" s="6">
-        <f t="shared" si="24"/>
-        <v>82</v>
-      </c>
-      <c r="AI49" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ49" s="3">
         <f t="shared" si="25"/>
         <v>82</v>
       </c>
+      <c r="AI49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ49" s="3">
+        <f t="shared" si="26"/>
+        <v>82</v>
+      </c>
       <c r="AK49" s="3" t="s">
         <v>60</v>
       </c>
@@ -10083,36 +10099,36 @@
         <v>2</v>
       </c>
       <c r="AM49" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>84</v>
       </c>
       <c r="AN49" s="3">
         <v>1</v>
       </c>
       <c r="AO49" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>85</v>
       </c>
       <c r="AP49" s="3">
         <v>3</v>
       </c>
       <c r="AQ49" s="3">
+        <f t="shared" si="31"/>
+        <v>88</v>
+      </c>
+      <c r="AR49" s="3">
+        <f t="shared" si="36"/>
+        <v>95</v>
+      </c>
+      <c r="AS49" s="3">
+        <f t="shared" si="29"/>
+        <v>102</v>
+      </c>
+      <c r="AT49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU49" s="3">
         <f t="shared" si="30"/>
-        <v>88</v>
-      </c>
-      <c r="AR49" s="3">
-        <f t="shared" si="35"/>
-        <v>95</v>
-      </c>
-      <c r="AS49" s="3">
-        <f t="shared" si="28"/>
-        <v>102</v>
-      </c>
-      <c r="AT49" s="3">
-        <v>0</v>
-      </c>
-      <c r="AU49" s="3">
-        <f t="shared" si="29"/>
         <v>15</v>
       </c>
       <c r="AV49" s="3" t="s">
@@ -10166,7 +10182,7 @@
         <v>7</v>
       </c>
       <c r="M50" s="3">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>9</v>
       </c>
       <c r="N50" s="3">
@@ -10177,33 +10193,33 @@
         <v>22</v>
       </c>
       <c r="P50" s="3">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>5</v>
       </c>
       <c r="Q50" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>26</v>
       </c>
       <c r="R50" s="3">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>23</v>
       </c>
       <c r="S50" s="3">
         <v>7</v>
       </c>
       <c r="T50" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U50" s="3">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>30</v>
       </c>
       <c r="V50" s="3">
         <v>2</v>
       </c>
       <c r="W50" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>31</v>
       </c>
       <c r="X50" s="3">
@@ -10218,7 +10234,7 @@
         <v>31</v>
       </c>
       <c r="AA50" s="6">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>34</v>
       </c>
       <c r="AB50" s="3">
@@ -10234,23 +10250,23 @@
         <v>48</v>
       </c>
       <c r="AF50" s="3">
-        <f t="shared" si="23"/>
-        <v>81</v>
-      </c>
-      <c r="AG50" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH50" s="6">
         <f t="shared" si="24"/>
         <v>81</v>
       </c>
-      <c r="AI50" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ50" s="3">
+      <c r="AG50" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH50" s="6">
         <f t="shared" si="25"/>
         <v>81</v>
       </c>
+      <c r="AI50" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ50" s="3">
+        <f t="shared" si="26"/>
+        <v>81</v>
+      </c>
       <c r="AK50" s="3" t="s">
         <v>60</v>
       </c>
@@ -10258,36 +10274,36 @@
         <v>3</v>
       </c>
       <c r="AM50" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>84</v>
       </c>
       <c r="AN50" s="3">
         <v>8</v>
       </c>
       <c r="AO50" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>92</v>
       </c>
       <c r="AP50" s="3">
         <v>0</v>
       </c>
       <c r="AQ50" s="3">
+        <f t="shared" si="31"/>
+        <v>92</v>
+      </c>
+      <c r="AR50" s="3">
+        <f t="shared" si="36"/>
+        <v>99</v>
+      </c>
+      <c r="AS50" s="3">
+        <f t="shared" si="29"/>
+        <v>106</v>
+      </c>
+      <c r="AT50" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU50" s="3">
         <f t="shared" si="30"/>
-        <v>92</v>
-      </c>
-      <c r="AR50" s="3">
-        <f t="shared" si="35"/>
-        <v>99</v>
-      </c>
-      <c r="AS50" s="3">
-        <f t="shared" si="28"/>
-        <v>106</v>
-      </c>
-      <c r="AT50" s="3">
-        <v>0</v>
-      </c>
-      <c r="AU50" s="3">
-        <f t="shared" si="29"/>
         <v>11</v>
       </c>
       <c r="AV50" s="3" t="s">
@@ -10341,7 +10357,7 @@
         <v>2</v>
       </c>
       <c r="M51" s="3">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>9</v>
       </c>
       <c r="N51" s="3">
@@ -10352,33 +10368,33 @@
         <v>22</v>
       </c>
       <c r="P51" s="3">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>5</v>
       </c>
       <c r="Q51" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>26</v>
       </c>
       <c r="R51" s="3">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>23</v>
       </c>
       <c r="S51" s="3">
         <v>7</v>
       </c>
       <c r="T51" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="U51" s="3">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>30</v>
       </c>
       <c r="V51" s="3">
         <v>2</v>
       </c>
       <c r="W51" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>31</v>
       </c>
       <c r="X51" s="3">
@@ -10393,7 +10409,7 @@
         <v>33</v>
       </c>
       <c r="AA51" s="6">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>34</v>
       </c>
       <c r="AB51" s="3">
@@ -10409,23 +10425,23 @@
         <v>50</v>
       </c>
       <c r="AF51" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>83</v>
       </c>
       <c r="AG51" s="6">
         <v>3</v>
       </c>
       <c r="AH51" s="6">
-        <f t="shared" si="24"/>
-        <v>86</v>
-      </c>
-      <c r="AI51" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ51" s="3">
         <f t="shared" si="25"/>
         <v>86</v>
       </c>
+      <c r="AI51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ51" s="3">
+        <f t="shared" si="26"/>
+        <v>86</v>
+      </c>
       <c r="AK51" s="3" t="s">
         <v>60</v>
       </c>
@@ -10433,36 +10449,36 @@
         <v>4</v>
       </c>
       <c r="AM51" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>90</v>
       </c>
       <c r="AN51" s="3">
         <v>2</v>
       </c>
       <c r="AO51" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>92</v>
       </c>
       <c r="AP51" s="3">
         <v>1</v>
       </c>
       <c r="AQ51" s="3">
+        <f t="shared" si="31"/>
+        <v>93</v>
+      </c>
+      <c r="AR51" s="3">
+        <f t="shared" si="36"/>
+        <v>100</v>
+      </c>
+      <c r="AS51" s="3">
+        <f t="shared" si="29"/>
+        <v>107</v>
+      </c>
+      <c r="AT51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU51" s="3">
         <f t="shared" si="30"/>
-        <v>93</v>
-      </c>
-      <c r="AR51" s="3">
-        <f t="shared" si="35"/>
-        <v>100</v>
-      </c>
-      <c r="AS51" s="3">
-        <f t="shared" si="28"/>
-        <v>107</v>
-      </c>
-      <c r="AT51" s="3">
-        <v>0</v>
-      </c>
-      <c r="AU51" s="3">
-        <f t="shared" si="29"/>
         <v>11</v>
       </c>
       <c r="AV51" s="3" t="s">
@@ -10516,7 +10532,7 @@
         <v>7</v>
       </c>
       <c r="M52" s="3">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>9</v>
       </c>
       <c r="N52" s="3">
@@ -10527,33 +10543,33 @@
         <v>15</v>
       </c>
       <c r="P52" s="3">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>5</v>
       </c>
       <c r="Q52" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>19</v>
       </c>
       <c r="R52" s="3">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>16</v>
       </c>
       <c r="S52" s="3">
         <v>3</v>
       </c>
       <c r="T52" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>18</v>
       </c>
       <c r="U52" s="3">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>19</v>
       </c>
       <c r="V52" s="3">
         <v>5</v>
       </c>
       <c r="W52" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>23</v>
       </c>
       <c r="X52" s="3">
@@ -10567,7 +10583,7 @@
         <v>23</v>
       </c>
       <c r="AA52" s="6">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>25</v>
       </c>
       <c r="AB52" s="3">
@@ -10583,21 +10599,21 @@
         <v>40</v>
       </c>
       <c r="AF52" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>64</v>
       </c>
       <c r="AG52" s="6">
         <v>3</v>
       </c>
       <c r="AH52" s="6">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>67</v>
       </c>
       <c r="AI52" s="3">
         <v>7</v>
       </c>
       <c r="AJ52" s="3">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>74</v>
       </c>
       <c r="AK52" s="3">
@@ -10607,36 +10623,36 @@
         <v>6</v>
       </c>
       <c r="AM52" s="3">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>80</v>
       </c>
       <c r="AN52" s="3">
         <v>2</v>
       </c>
       <c r="AO52" s="3">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>82</v>
       </c>
       <c r="AP52" s="3">
         <v>0</v>
       </c>
       <c r="AQ52" s="3">
+        <f t="shared" si="31"/>
+        <v>82</v>
+      </c>
+      <c r="AR52" s="3">
+        <f t="shared" si="36"/>
+        <v>89</v>
+      </c>
+      <c r="AS52" s="3">
+        <f t="shared" si="29"/>
+        <v>96</v>
+      </c>
+      <c r="AT52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU52" s="3">
         <f t="shared" si="30"/>
-        <v>82</v>
-      </c>
-      <c r="AR52" s="3">
-        <f t="shared" si="35"/>
-        <v>89</v>
-      </c>
-      <c r="AS52" s="3">
-        <f t="shared" si="28"/>
-        <v>96</v>
-      </c>
-      <c r="AT52" s="3">
-        <v>0</v>
-      </c>
-      <c r="AU52" s="3">
-        <f t="shared" si="29"/>
         <v>9</v>
       </c>
       <c r="AV52" s="3" t="s">
@@ -10654,25 +10670,25 @@
     </row>
     <row r="53" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="B53" s="38" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="C53" s="39" t="s">
         <v>68</v>
       </c>
       <c r="D53" s="38" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E53" s="38" t="s">
         <v>81</v>
       </c>
       <c r="F53" s="19">
-        <v>90014400</v>
+        <v>91017700</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H53" s="2">
         <v>0</v>
@@ -10690,7 +10706,7 @@
         <v>5</v>
       </c>
       <c r="M53" s="3">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>9</v>
       </c>
       <c r="N53" s="23">
@@ -10704,40 +10720,39 @@
         <v>5</v>
       </c>
       <c r="Q53" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>14</v>
       </c>
       <c r="R53" s="23">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S53" s="23">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="T53" s="25">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="U53" s="23">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="V53" s="23">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="W53" s="23">
-        <f t="shared" si="22"/>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="X53" s="23">
         <v>1</v>
       </c>
       <c r="Y53" s="3">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="Z53" s="6">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="AA53" s="6">
-        <f t="shared" si="36"/>
-        <v>22</v>
+        <f t="shared" si="37"/>
+        <v>25</v>
       </c>
       <c r="AB53" s="23">
         <v>4</v>
@@ -10745,62 +10760,62 @@
       <c r="AC53" s="23"/>
       <c r="AD53" s="23"/>
       <c r="AE53" s="23">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="AF53" s="23">
-        <f t="shared" si="23"/>
-        <v>67</v>
+        <f t="shared" si="24"/>
+        <v>63</v>
       </c>
       <c r="AG53" s="23">
         <v>3</v>
       </c>
       <c r="AH53" s="23">
-        <f t="shared" si="24"/>
-        <v>70</v>
+        <f t="shared" si="25"/>
+        <v>66</v>
       </c>
       <c r="AI53" s="23">
         <v>7</v>
       </c>
       <c r="AJ53" s="23">
-        <f t="shared" si="25"/>
-        <v>77</v>
+        <f t="shared" si="26"/>
+        <v>73</v>
       </c>
       <c r="AK53" s="23"/>
-      <c r="AL53" s="23">
-        <v>3</v>
+      <c r="AL53" s="47">
+        <v>2</v>
       </c>
       <c r="AM53" s="23">
-        <f t="shared" si="26"/>
-        <v>80</v>
+        <f t="shared" si="27"/>
+        <v>75</v>
       </c>
       <c r="AN53" s="23">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AO53" s="23">
-        <f t="shared" si="27"/>
-        <v>82</v>
+        <f t="shared" si="28"/>
+        <v>83</v>
       </c>
       <c r="AP53" s="23">
         <v>2</v>
       </c>
       <c r="AQ53" s="23">
-        <f t="shared" si="30"/>
-        <v>84</v>
+        <f t="shared" si="31"/>
+        <v>85</v>
       </c>
       <c r="AR53" s="23">
-        <f t="shared" si="35"/>
-        <v>91</v>
+        <f t="shared" si="36"/>
+        <v>92</v>
       </c>
       <c r="AS53" s="23">
-        <f t="shared" si="28"/>
-        <v>112</v>
+        <f t="shared" si="29"/>
+        <v>113</v>
       </c>
       <c r="AT53" s="23">
         <v>14</v>
       </c>
       <c r="AU53" s="3">
-        <f t="shared" si="29"/>
-        <v>22</v>
+        <f t="shared" si="30"/>
+        <v>15</v>
       </c>
       <c r="AV53" s="23" t="s">
         <v>133</v>
@@ -10811,31 +10826,31 @@
       <c r="AX53" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="AY53" s="37">
-        <v>46143</v>
+      <c r="AY53" s="21">
+        <v>46507</v>
       </c>
     </row>
-    <row r="54" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B54" s="38" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="C54" s="39" t="s">
         <v>68</v>
       </c>
       <c r="D54" s="38" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="E54" s="38" t="s">
         <v>81</v>
       </c>
       <c r="F54" s="19">
-        <v>91017700</v>
+        <v>90014400</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H54" s="2">
         <v>0</v>
@@ -10853,7 +10868,7 @@
         <v>5</v>
       </c>
       <c r="M54" s="3">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>9</v>
       </c>
       <c r="N54" s="23">
@@ -10867,39 +10882,40 @@
         <v>5</v>
       </c>
       <c r="Q54" s="3">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>14</v>
       </c>
       <c r="R54" s="23">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S54" s="23">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="T54" s="25">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="U54" s="23">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="V54" s="23">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="W54" s="23">
-        <v>22</v>
+        <f>+U54+V54-1</f>
+        <v>18</v>
       </c>
       <c r="X54" s="23">
         <v>1</v>
       </c>
       <c r="Y54" s="3">
+        <v>18</v>
+      </c>
+      <c r="Z54" s="6">
+        <v>19</v>
+      </c>
+      <c r="AA54" s="6">
+        <f t="shared" si="37"/>
         <v>22</v>
-      </c>
-      <c r="Z54" s="6">
-        <v>22</v>
-      </c>
-      <c r="AA54" s="6">
-        <f t="shared" si="36"/>
-        <v>25</v>
       </c>
       <c r="AB54" s="23">
         <v>4</v>
@@ -10907,62 +10923,62 @@
       <c r="AC54" s="23"/>
       <c r="AD54" s="23"/>
       <c r="AE54" s="23">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="AF54" s="23">
-        <f t="shared" si="23"/>
-        <v>63</v>
+        <f t="shared" si="24"/>
+        <v>67</v>
       </c>
       <c r="AG54" s="23">
         <v>3</v>
       </c>
       <c r="AH54" s="23">
-        <f t="shared" si="24"/>
-        <v>66</v>
+        <f t="shared" si="25"/>
+        <v>70</v>
       </c>
       <c r="AI54" s="23">
         <v>7</v>
       </c>
       <c r="AJ54" s="23">
-        <f t="shared" si="25"/>
-        <v>73</v>
+        <f t="shared" si="26"/>
+        <v>77</v>
       </c>
       <c r="AK54" s="23"/>
-      <c r="AL54" s="47">
+      <c r="AL54" s="23">
+        <v>3</v>
+      </c>
+      <c r="AM54" s="23">
+        <f t="shared" si="27"/>
+        <v>80</v>
+      </c>
+      <c r="AN54" s="23">
         <v>2</v>
       </c>
-      <c r="AM54" s="23">
-        <f t="shared" si="26"/>
-        <v>75</v>
-      </c>
-      <c r="AN54" s="23">
-        <v>8</v>
-      </c>
       <c r="AO54" s="23">
-        <f t="shared" si="27"/>
-        <v>83</v>
+        <f t="shared" si="28"/>
+        <v>82</v>
       </c>
       <c r="AP54" s="23">
         <v>2</v>
       </c>
       <c r="AQ54" s="23">
-        <f t="shared" si="30"/>
-        <v>85</v>
+        <f t="shared" si="31"/>
+        <v>84</v>
       </c>
       <c r="AR54" s="23">
-        <f t="shared" si="35"/>
-        <v>92</v>
+        <f t="shared" si="36"/>
+        <v>91</v>
       </c>
       <c r="AS54" s="23">
-        <f t="shared" si="28"/>
-        <v>113</v>
+        <f t="shared" si="29"/>
+        <v>112</v>
       </c>
       <c r="AT54" s="23">
         <v>14</v>
       </c>
       <c r="AU54" s="3">
-        <f t="shared" si="29"/>
-        <v>15</v>
+        <f t="shared" si="30"/>
+        <v>22</v>
       </c>
       <c r="AV54" s="23" t="s">
         <v>133</v>
@@ -10973,7 +10989,486 @@
       <c r="AX54" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="AY54" s="21">
+      <c r="AY54" s="37">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="55" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="B55" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="C55" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="D55" s="43" t="s">
+        <v>136</v>
+      </c>
+      <c r="E55" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="F55" s="19">
+        <v>90016500</v>
+      </c>
+      <c r="G55" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="H55" s="2">
+        <v>0</v>
+      </c>
+      <c r="I55" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="J55" s="2">
+        <v>29159</v>
+      </c>
+      <c r="K55" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="L55" s="3">
+        <v>8</v>
+      </c>
+      <c r="M55" s="3">
+        <v>0</v>
+      </c>
+      <c r="N55" s="3">
+        <v>14</v>
+      </c>
+      <c r="O55" s="3">
+        <v>8</v>
+      </c>
+      <c r="P55" s="3">
+        <v>7</v>
+      </c>
+      <c r="Q55" s="3">
+        <f t="shared" si="21"/>
+        <v>14</v>
+      </c>
+      <c r="R55" s="3">
+        <v>15</v>
+      </c>
+      <c r="S55" s="3">
+        <v>7</v>
+      </c>
+      <c r="T55" s="3">
+        <v>21</v>
+      </c>
+      <c r="U55" s="3">
+        <f>+T55+1</f>
+        <v>22</v>
+      </c>
+      <c r="V55" s="3">
+        <v>7</v>
+      </c>
+      <c r="W55" s="3">
+        <f>+U55+V55-1</f>
+        <v>28</v>
+      </c>
+      <c r="X55" s="3">
+        <v>2</v>
+      </c>
+      <c r="Y55" s="3">
+        <v>28</v>
+      </c>
+      <c r="Z55" s="6">
+        <v>28</v>
+      </c>
+      <c r="AA55" s="6">
+        <v>29</v>
+      </c>
+      <c r="AB55" s="3">
+        <v>6</v>
+      </c>
+      <c r="AC55" s="3">
+        <v>7</v>
+      </c>
+      <c r="AD55" s="3">
+        <v>7</v>
+      </c>
+      <c r="AE55" s="3">
+        <v>50</v>
+      </c>
+      <c r="AF55" s="3">
+        <f t="shared" si="24"/>
+        <v>78</v>
+      </c>
+      <c r="AG55" s="6">
+        <v>3</v>
+      </c>
+      <c r="AH55" s="6">
+        <f t="shared" si="25"/>
+        <v>81</v>
+      </c>
+      <c r="AI55" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ55" s="3">
+        <f t="shared" si="26"/>
+        <v>81</v>
+      </c>
+      <c r="AK55" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL55" s="46">
+        <v>10</v>
+      </c>
+      <c r="AM55" s="3">
+        <f t="shared" si="27"/>
+        <v>91</v>
+      </c>
+      <c r="AN55" s="3">
+        <v>5</v>
+      </c>
+      <c r="AO55" s="3">
+        <f t="shared" si="28"/>
+        <v>96</v>
+      </c>
+      <c r="AP55" s="3">
+        <v>3</v>
+      </c>
+      <c r="AQ55" s="3">
+        <f t="shared" si="31"/>
+        <v>99</v>
+      </c>
+      <c r="AR55" s="3">
+        <f t="shared" si="36"/>
+        <v>106</v>
+      </c>
+      <c r="AS55" s="3">
+        <f t="shared" si="29"/>
+        <v>113</v>
+      </c>
+      <c r="AT55" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU55" s="3">
+        <f t="shared" si="30"/>
+        <v>14</v>
+      </c>
+      <c r="AV55" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="AW55" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="AX55" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="AY55" s="40">
+        <v>46507</v>
+      </c>
+    </row>
+    <row r="56" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E56" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="F56" s="19">
+        <v>91017700</v>
+      </c>
+      <c r="G56" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="H56" s="2">
+        <v>222222</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="J56" s="2">
+        <v>222222</v>
+      </c>
+      <c r="K56" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="L56" s="3">
+        <v>7</v>
+      </c>
+      <c r="M56" s="3">
+        <v>9</v>
+      </c>
+      <c r="N56" s="23">
+        <v>21</v>
+      </c>
+      <c r="O56" s="3">
+        <v>29</v>
+      </c>
+      <c r="P56" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q56" s="3">
+        <v>33</v>
+      </c>
+      <c r="R56" s="23">
+        <v>30</v>
+      </c>
+      <c r="S56" s="23">
+        <v>7</v>
+      </c>
+      <c r="T56" s="23">
+        <v>36</v>
+      </c>
+      <c r="U56" s="23">
+        <v>37</v>
+      </c>
+      <c r="V56" s="23">
+        <v>1</v>
+      </c>
+      <c r="W56" s="23">
+        <v>37</v>
+      </c>
+      <c r="X56" s="23">
+        <v>0</v>
+      </c>
+      <c r="Y56" s="3">
+        <v>37</v>
+      </c>
+      <c r="Z56" s="6">
+        <v>42</v>
+      </c>
+      <c r="AA56" s="6">
+        <v>44</v>
+      </c>
+      <c r="AB56" s="23">
+        <v>3</v>
+      </c>
+      <c r="AC56" s="33">
+        <v>4</v>
+      </c>
+      <c r="AD56" s="23">
+        <v>4</v>
+      </c>
+      <c r="AE56" s="23">
+        <v>40</v>
+      </c>
+      <c r="AF56" s="23">
+        <v>83</v>
+      </c>
+      <c r="AG56" s="23">
+        <v>3</v>
+      </c>
+      <c r="AH56" s="23">
+        <v>86</v>
+      </c>
+      <c r="AI56" s="23">
+        <v>0</v>
+      </c>
+      <c r="AJ56" s="23">
+        <v>86</v>
+      </c>
+      <c r="AK56" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL56" s="23">
+        <v>2</v>
+      </c>
+      <c r="AM56" s="23">
+        <f t="shared" si="27"/>
+        <v>88</v>
+      </c>
+      <c r="AN56" s="23">
+        <v>1</v>
+      </c>
+      <c r="AO56" s="23">
+        <f t="shared" si="28"/>
+        <v>89</v>
+      </c>
+      <c r="AP56" s="23">
+        <v>3</v>
+      </c>
+      <c r="AQ56" s="23">
+        <f t="shared" si="31"/>
+        <v>92</v>
+      </c>
+      <c r="AR56" s="23">
+        <f t="shared" si="36"/>
+        <v>99</v>
+      </c>
+      <c r="AS56" s="23">
+        <f t="shared" ref="AS56:AS57" si="38">+AR56+7+AT56</f>
+        <v>106</v>
+      </c>
+      <c r="AT56" s="23">
+        <v>0</v>
+      </c>
+      <c r="AU56" s="23">
+        <v>14</v>
+      </c>
+      <c r="AV56" s="20" t="s">
+        <v>130</v>
+      </c>
+      <c r="AW56" s="40" t="s">
+        <v>131</v>
+      </c>
+      <c r="AX56" t="s">
+        <v>75</v>
+      </c>
+      <c r="AY56">
+        <v>46507</v>
+      </c>
+    </row>
+    <row r="57" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="B57" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F57" s="19">
+        <v>90016500</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="H57" s="2">
+        <v>0</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="J57" s="2">
+        <v>29159</v>
+      </c>
+      <c r="K57" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="L57" s="3">
+        <v>5</v>
+      </c>
+      <c r="M57" s="3">
+        <v>8</v>
+      </c>
+      <c r="N57" s="3">
+        <v>1</v>
+      </c>
+      <c r="O57" s="3">
+        <v>8</v>
+      </c>
+      <c r="P57" s="3">
+        <v>6</v>
+      </c>
+      <c r="Q57" s="3">
+        <v>13</v>
+      </c>
+      <c r="R57" s="3">
+        <v>9</v>
+      </c>
+      <c r="S57" s="3">
+        <v>12</v>
+      </c>
+      <c r="T57" s="3">
+        <v>20</v>
+      </c>
+      <c r="U57" s="3">
+        <v>22</v>
+      </c>
+      <c r="V57" s="3">
+        <v>5</v>
+      </c>
+      <c r="W57" s="3">
+        <v>26</v>
+      </c>
+      <c r="X57" s="3">
+        <v>4</v>
+      </c>
+      <c r="Y57" s="3">
+        <v>29</v>
+      </c>
+      <c r="Z57" s="6">
+        <v>34</v>
+      </c>
+      <c r="AA57" s="6">
+        <v>36</v>
+      </c>
+      <c r="AB57" s="3">
+        <v>4</v>
+      </c>
+      <c r="AC57" s="3"/>
+      <c r="AD57" s="3"/>
+      <c r="AE57" s="6">
+        <v>34</v>
+      </c>
+      <c r="AF57" s="6">
+        <v>69</v>
+      </c>
+      <c r="AG57" s="3">
+        <v>3</v>
+      </c>
+      <c r="AH57" s="3">
+        <v>72</v>
+      </c>
+      <c r="AI57" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ57" s="3">
+        <v>72</v>
+      </c>
+      <c r="AK57" s="3"/>
+      <c r="AL57" s="3">
+        <v>2</v>
+      </c>
+      <c r="AM57" s="3">
+        <v>74</v>
+      </c>
+      <c r="AN57" s="3">
+        <v>1</v>
+      </c>
+      <c r="AO57" s="3">
+        <v>75</v>
+      </c>
+      <c r="AP57" s="3">
+        <v>3</v>
+      </c>
+      <c r="AQ57" s="23">
+        <f t="shared" si="31"/>
+        <v>78</v>
+      </c>
+      <c r="AR57" s="23">
+        <f t="shared" si="36"/>
+        <v>85</v>
+      </c>
+      <c r="AS57" s="23">
+        <f t="shared" si="38"/>
+        <v>106</v>
+      </c>
+      <c r="AT57" s="3">
+        <v>14</v>
+      </c>
+      <c r="AU57" s="3">
+        <v>27</v>
+      </c>
+      <c r="AV57" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="AW57" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="AX57" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY57">
         <v>46507</v>
       </c>
     </row>
@@ -11000,26 +11495,19 @@
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
-  <autoFilter ref="A1:AY54" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
-    <filterColumn colId="3">
+  <autoFilter ref="A1:AY57" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
+    <filterColumn colId="0">
       <filters>
-        <filter val="ESALG"/>
-        <filter val="ESVLC"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="47">
-      <filters>
-        <filter val="Direct"/>
-        <filter val="Indirect"/>
+        <filter val="930"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <phoneticPr fontId="8" type="noConversion"/>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:E12 K2:K12 C53:C1048195 E53:E1048195 D53:D60 D72:D1048195 C16:E52 K16:K1048195" xr:uid="{833F6030-824F-4AAE-BA3C-131D886541AF}">
+  <dataValidations disablePrompts="1" count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:E12 K2:K12 C58:C1048195 D72:D1048195 C16:E57 E58:E1048195 D58:D60 K16:K1048195" xr:uid="{833F6030-824F-4AAE-BA3C-131D886541AF}">
       <formula1>shippername</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J10 H55:K1048195 C53:C1048195 E53:E1048195 D53:D60 D72:D1048195 C2:E52 J12:J54 I2:I54 K2:K54" xr:uid="{DD2A48DC-7068-4BD6-8A6F-E802386CE572}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J10 D58:D60 H58:K1048195 C58:C1048195 E58:E1048195 D72:D1048195 J12:J57 I2:I57 C2:E57 K2:K57" xr:uid="{DD2A48DC-7068-4BD6-8A6F-E802386CE572}">
       <formula1>AILNname</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Please check information" error="This is not a known plant, please check the spelling or enter the information in the sheet &quot;Plant_ALIN&quot;" sqref="G2:G1048195" xr:uid="{D2D52A73-EC4B-4324-8BC4-BD77EF4C5461}">

</xml_diff>